<commit_message>
FIx doc file excel test
</commit_message>
<xml_diff>
--- a/maHĐ.xlsx
+++ b/maHĐ.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$151</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -27,14 +30,29 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="447">
   <si>
     <t>MÃ KHÁCH HÀNG</t>
   </si>
   <si>
+    <t>EVN</t>
+  </si>
+  <si>
     <t>SỐ TIỀN</t>
   </si>
   <si>
+    <t>HẠN THANH TOÁN</t>
+  </si>
+  <si>
+    <t>PC03PP0243527</t>
+  </si>
+  <si>
+    <t>EVNCPC</t>
+  </si>
+  <si>
+    <t>80.751.276</t>
+  </si>
+  <si>
     <t>PC03GG0718405</t>
   </si>
   <si>
@@ -119,10 +137,7 @@
     <t>11.254.384</t>
   </si>
   <si>
-    <t>8.360.029</t>
-  </si>
-  <si>
-    <t>12.157.893</t>
+    <t>17/03/2026</t>
   </si>
   <si>
     <t>PC08BB0252277</t>
@@ -155,19 +170,13 @@
     <t>18.624.481</t>
   </si>
   <si>
-    <t>16.442.603</t>
-  </si>
-  <si>
-    <t>16.464.699</t>
-  </si>
-  <si>
     <t>PC03DD0479701</t>
   </si>
   <si>
     <t>53.589.442</t>
   </si>
   <si>
-    <t>56.474.021</t>
+    <t>23/03/2026</t>
   </si>
   <si>
     <t>PC08FF0619324</t>
@@ -182,21 +191,21 @@
     <t>55.393.928</t>
   </si>
   <si>
-    <t>45.219.172</t>
-  </si>
-  <si>
-    <t>54.421.040</t>
-  </si>
-  <si>
     <t>PD27007696347</t>
   </si>
   <si>
+    <t>EVNHANOI</t>
+  </si>
+  <si>
     <t>239.728.637</t>
   </si>
   <si>
     <t>PA22040530046</t>
   </si>
   <si>
+    <t>EVNNCP</t>
+  </si>
+  <si>
     <t>99.625.896</t>
   </si>
   <si>
@@ -206,9 +215,6 @@
     <t>10.795.162</t>
   </si>
   <si>
-    <t>13.991.875</t>
-  </si>
-  <si>
     <t>PA25VT0039197</t>
   </si>
   <si>
@@ -239,7 +245,7 @@
     <t>125.086.291</t>
   </si>
   <si>
-    <t>131.207.558</t>
+    <t>22/03/2026</t>
   </si>
   <si>
     <t>PA02PT0024884</t>
@@ -254,9 +260,6 @@
     <t>94.018.061</t>
   </si>
   <si>
-    <t>104.195.462</t>
-  </si>
-  <si>
     <t>PA25BX0025561</t>
   </si>
   <si>
@@ -323,7 +326,7 @@
     <t>77.948.158</t>
   </si>
   <si>
-    <t>103.157.911</t>
+    <t>20/03/2026</t>
   </si>
   <si>
     <t>PNTD003012612</t>
@@ -368,9 +371,6 @@
     <t>63.630.440</t>
   </si>
   <si>
-    <t>71.899.015</t>
-  </si>
-  <si>
     <t>PC02DD0552944</t>
   </si>
   <si>
@@ -389,12 +389,6 @@
     <t>4.514.078</t>
   </si>
   <si>
-    <t>2.808.287</t>
-  </si>
-  <si>
-    <t>4.759.039</t>
-  </si>
-  <si>
     <t>PC01EE0573816</t>
   </si>
   <si>
@@ -557,9 +551,6 @@
     <t>20.405.084</t>
   </si>
   <si>
-    <t>65.658.440</t>
-  </si>
-  <si>
     <t>PC02KK0924548</t>
   </si>
   <si>
@@ -641,6 +632,9 @@
     <t>PB16060029755</t>
   </si>
   <si>
+    <t>EVNSPC</t>
+  </si>
+  <si>
     <t>4.837.085</t>
   </si>
   <si>
@@ -662,7 +656,7 @@
     <t>141.697.728</t>
   </si>
   <si>
-    <t>308.785.427</t>
+    <t>19/03/2026</t>
   </si>
   <si>
     <t>PA04TP1480282</t>
@@ -671,27 +665,12 @@
     <t>87.951.744</t>
   </si>
   <si>
-    <t>105.165.475</t>
-  </si>
-  <si>
     <t>PA18LC0108438</t>
   </si>
   <si>
     <t>116.694.432</t>
   </si>
   <si>
-    <t>PNNB000047048</t>
-  </si>
-  <si>
-    <t>316.974.643</t>
-  </si>
-  <si>
-    <t>199.974.643</t>
-  </si>
-  <si>
-    <t>342.588.604</t>
-  </si>
-  <si>
     <t>PA11CL0030910</t>
   </si>
   <si>
@@ -716,7 +695,7 @@
     <t>79.292.736</t>
   </si>
   <si>
-    <t>79.320.038</t>
+    <t>24/03/2026</t>
   </si>
   <si>
     <t>PM01009091017</t>
@@ -725,16 +704,13 @@
     <t>68.788.570</t>
   </si>
   <si>
-    <t>85.945.795</t>
-  </si>
-  <si>
     <t>PM13000373400</t>
   </si>
   <si>
     <t>169.010.323</t>
   </si>
   <si>
-    <t>188.830.310</t>
+    <t>21/03/2026</t>
   </si>
   <si>
     <t>PA05090091270</t>
@@ -755,9 +731,6 @@
     <t>78.624.756</t>
   </si>
   <si>
-    <t>79.512.732</t>
-  </si>
-  <si>
     <t>PA17LS0033396</t>
   </si>
   <si>
@@ -782,9 +755,6 @@
     <t>151.670.448</t>
   </si>
   <si>
-    <t>172.592.424</t>
-  </si>
-  <si>
     <t>PM21000062233</t>
   </si>
   <si>
@@ -809,9 +779,6 @@
     <t>105.721.718</t>
   </si>
   <si>
-    <t>119.741.818</t>
-  </si>
-  <si>
     <t>PA18VB0028340</t>
   </si>
   <si>
@@ -836,12 +803,6 @@
     <t>17.921.088</t>
   </si>
   <si>
-    <t>12.329.626</t>
-  </si>
-  <si>
-    <t>14.354.150</t>
-  </si>
-  <si>
     <t>PA02DH1026489</t>
   </si>
   <si>
@@ -876,6 +837,540 @@
   </si>
   <si>
     <t>64.376.208</t>
+  </si>
+  <si>
+    <t>PA02YL0029500</t>
+  </si>
+  <si>
+    <t>92.848.872</t>
+  </si>
+  <si>
+    <t>PA02TN0034159</t>
+  </si>
+  <si>
+    <t>104.010.048</t>
+  </si>
+  <si>
+    <t>PA02TN0034414</t>
+  </si>
+  <si>
+    <t>45.130.694</t>
+  </si>
+  <si>
+    <t>PA02TT0041868</t>
+  </si>
+  <si>
+    <t>126.433.267</t>
+  </si>
+  <si>
+    <t>PA02TT0044820</t>
+  </si>
+  <si>
+    <t>140.470.157</t>
+  </si>
+  <si>
+    <t>PA02LT0016984</t>
+  </si>
+  <si>
+    <t>160.788.672</t>
+  </si>
+  <si>
+    <t>PA02LT0017753</t>
+  </si>
+  <si>
+    <t>85.598.986</t>
+  </si>
+  <si>
+    <t>PA02LT0017786</t>
+  </si>
+  <si>
+    <t>88.349.184</t>
+  </si>
+  <si>
+    <t>PA02HH0036488</t>
+  </si>
+  <si>
+    <t>34.197.811</t>
+  </si>
+  <si>
+    <t>PA02HH0040202</t>
+  </si>
+  <si>
+    <t>27.846.374</t>
+  </si>
+  <si>
+    <t>PA02HH0042655</t>
+  </si>
+  <si>
+    <t>10.809.504</t>
+  </si>
+  <si>
+    <t>PA02HH0043104</t>
+  </si>
+  <si>
+    <t>25.997.760</t>
+  </si>
+  <si>
+    <t>PA02HH0043143</t>
+  </si>
+  <si>
+    <t>145.769.976</t>
+  </si>
+  <si>
+    <t>PA29020025651</t>
+  </si>
+  <si>
+    <t>86.805.043</t>
+  </si>
+  <si>
+    <t>PA29010022064</t>
+  </si>
+  <si>
+    <t>37.572.077</t>
+  </si>
+  <si>
+    <t>PA29010022062</t>
+  </si>
+  <si>
+    <t>20.047.565</t>
+  </si>
+  <si>
+    <t>PA29010022063</t>
+  </si>
+  <si>
+    <t>42.603.494</t>
+  </si>
+  <si>
+    <t>PA29010021429</t>
+  </si>
+  <si>
+    <t>26.916.138</t>
+  </si>
+  <si>
+    <t>PA10020328445</t>
+  </si>
+  <si>
+    <t>83.873.750</t>
+  </si>
+  <si>
+    <t>PA10020329686</t>
+  </si>
+  <si>
+    <t>26.556.595</t>
+  </si>
+  <si>
+    <t>PA10020329905</t>
+  </si>
+  <si>
+    <t>133.479.891</t>
+  </si>
+  <si>
+    <t>PB11020077036</t>
+  </si>
+  <si>
+    <t>138.051.065</t>
+  </si>
+  <si>
+    <t>PB11070059740</t>
+  </si>
+  <si>
+    <t>36.817.680</t>
+  </si>
+  <si>
+    <t>PB11020077039</t>
+  </si>
+  <si>
+    <t>74.046.882</t>
+  </si>
+  <si>
+    <t>PB09020086057</t>
+  </si>
+  <si>
+    <t>109.101.205</t>
+  </si>
+  <si>
+    <t>PNKS000136665</t>
+  </si>
+  <si>
+    <t>186.947.775</t>
+  </si>
+  <si>
+    <t>PE10000278727</t>
+  </si>
+  <si>
+    <t>EVNHCM</t>
+  </si>
+  <si>
+    <t>15.142.254</t>
+  </si>
+  <si>
+    <t>PK07000199578</t>
+  </si>
+  <si>
+    <t>7.552.373</t>
+  </si>
+  <si>
+    <t>PE01000134913</t>
+  </si>
+  <si>
+    <t>148.257.253</t>
+  </si>
+  <si>
+    <t>PP08000957588</t>
+  </si>
+  <si>
+    <t>53.595.808</t>
+  </si>
+  <si>
+    <t>15/03/2026</t>
+  </si>
+  <si>
+    <t>PP08000957769</t>
+  </si>
+  <si>
+    <t>59.792.729</t>
+  </si>
+  <si>
+    <t>PA25VY0071755</t>
+  </si>
+  <si>
+    <t>115.717.594</t>
+  </si>
+  <si>
+    <t>PA25TM0048571</t>
+  </si>
+  <si>
+    <t>107.440.819</t>
+  </si>
+  <si>
+    <t>PNYK000052011</t>
+  </si>
+  <si>
+    <t>85.721.544</t>
+  </si>
+  <si>
+    <t>PC03CC0030584</t>
+  </si>
+  <si>
+    <t>14.320.662</t>
+  </si>
+  <si>
+    <t>PC03BB0252696</t>
+  </si>
+  <si>
+    <t>120.128.486</t>
+  </si>
+  <si>
+    <t>PB09010084064</t>
+  </si>
+  <si>
+    <t>80.764.111</t>
+  </si>
+  <si>
+    <t>PB09010084065</t>
+  </si>
+  <si>
+    <t>90.546.373</t>
+  </si>
+  <si>
+    <t>PB14040069969</t>
+  </si>
+  <si>
+    <t>20.209.232</t>
+  </si>
+  <si>
+    <t>PB14040071353</t>
+  </si>
+  <si>
+    <t>74.977.667</t>
+  </si>
+  <si>
+    <t>PB06030117011</t>
+  </si>
+  <si>
+    <t>22.888.254</t>
+  </si>
+  <si>
+    <t>PB06030117044</t>
+  </si>
+  <si>
+    <t>43.914.658</t>
+  </si>
+  <si>
+    <t>PB06030117047</t>
+  </si>
+  <si>
+    <t>26.723.153</t>
+  </si>
+  <si>
+    <t>PB06030118340</t>
+  </si>
+  <si>
+    <t>112.415.979</t>
+  </si>
+  <si>
+    <t>PE16000375479</t>
+  </si>
+  <si>
+    <t>99.326.062</t>
+  </si>
+  <si>
+    <t>PE16000376253</t>
+  </si>
+  <si>
+    <t>101.883.032</t>
+  </si>
+  <si>
+    <t>PA09010245489</t>
+  </si>
+  <si>
+    <t>46.487.032</t>
+  </si>
+  <si>
+    <t>PB05060063421</t>
+  </si>
+  <si>
+    <t>51.333.517</t>
+  </si>
+  <si>
+    <t>PQ11000529289</t>
+  </si>
+  <si>
+    <t>11.128.320</t>
+  </si>
+  <si>
+    <t>PQ11000529196</t>
+  </si>
+  <si>
+    <t>48.428.833</t>
+  </si>
+  <si>
+    <t>PQ06000626200</t>
+  </si>
+  <si>
+    <t>45.253.356</t>
+  </si>
+  <si>
+    <t>PP03000966767</t>
+  </si>
+  <si>
+    <t>1.554.206</t>
+  </si>
+  <si>
+    <t>PNNQ003532279</t>
+  </si>
+  <si>
+    <t>60.601.383</t>
+  </si>
+  <si>
+    <t>PNNQ003532150</t>
+  </si>
+  <si>
+    <t>66.588.534</t>
+  </si>
+  <si>
+    <t>PNNQ003531890</t>
+  </si>
+  <si>
+    <t>143.579.254</t>
+  </si>
+  <si>
+    <t>PM23000092476</t>
+  </si>
+  <si>
+    <t>132.036.912</t>
+  </si>
+  <si>
+    <t>PM21000061960</t>
+  </si>
+  <si>
+    <t>113.836.579</t>
+  </si>
+  <si>
+    <t>PM21000061284</t>
+  </si>
+  <si>
+    <t>107.761.402</t>
+  </si>
+  <si>
+    <t>PM19000016004</t>
+  </si>
+  <si>
+    <t>124.604.179</t>
+  </si>
+  <si>
+    <t>PM17000099894</t>
+  </si>
+  <si>
+    <t>108.732.326</t>
+  </si>
+  <si>
+    <t>PM07000055838</t>
+  </si>
+  <si>
+    <t>137.550.744</t>
+  </si>
+  <si>
+    <t>PM05000019758</t>
+  </si>
+  <si>
+    <t>49.904.294</t>
+  </si>
+  <si>
+    <t>PM03000069761</t>
+  </si>
+  <si>
+    <t>101.034.734</t>
+  </si>
+  <si>
+    <t>PH14000006785</t>
+  </si>
+  <si>
+    <t>62.377.344</t>
+  </si>
+  <si>
+    <t>16/03/2026</t>
+  </si>
+  <si>
+    <t>PH11000731714</t>
+  </si>
+  <si>
+    <t>210.458.736</t>
+  </si>
+  <si>
+    <t>PH11000731682</t>
+  </si>
+  <si>
+    <t>25.766.554</t>
+  </si>
+  <si>
+    <t>PH10000023640</t>
+  </si>
+  <si>
+    <t>107.774.842</t>
+  </si>
+  <si>
+    <t>PH09000049549</t>
+  </si>
+  <si>
+    <t>57.558.470</t>
+  </si>
+  <si>
+    <t>PH04000073400</t>
+  </si>
+  <si>
+    <t>32.410.195</t>
+  </si>
+  <si>
+    <t>PE15000404717</t>
+  </si>
+  <si>
+    <t>132.410.637</t>
+  </si>
+  <si>
+    <t>PE15000403394</t>
+  </si>
+  <si>
+    <t>19.379.650</t>
+  </si>
+  <si>
+    <t>PE15000403346</t>
+  </si>
+  <si>
+    <t>45.081.092</t>
+  </si>
+  <si>
+    <t>PE15000403226</t>
+  </si>
+  <si>
+    <t>36.717.149</t>
+  </si>
+  <si>
+    <t>PE11002070284</t>
+  </si>
+  <si>
+    <t>55.378.817</t>
+  </si>
+  <si>
+    <t>PE11002069978</t>
+  </si>
+  <si>
+    <t>84.546.236</t>
+  </si>
+  <si>
+    <t>PE10000277229</t>
+  </si>
+  <si>
+    <t>PE10000276176</t>
+  </si>
+  <si>
+    <t>225.678.614</t>
+  </si>
+  <si>
+    <t>PE10000275961</t>
+  </si>
+  <si>
+    <t>150.597.516</t>
+  </si>
+  <si>
+    <t>PE10000275713</t>
+  </si>
+  <si>
+    <t>147.347.813</t>
+  </si>
+  <si>
+    <t>PE10000273214</t>
+  </si>
+  <si>
+    <t>101.792.484</t>
+  </si>
+  <si>
+    <t>PE10000270053</t>
+  </si>
+  <si>
+    <t>131.006.786</t>
+  </si>
+  <si>
+    <t>PE10000269648</t>
+  </si>
+  <si>
+    <t>61.326.677</t>
+  </si>
+  <si>
+    <t>PE08000347173</t>
+  </si>
+  <si>
+    <t>175.684.339</t>
+  </si>
+  <si>
+    <t>PE08000347113</t>
+  </si>
+  <si>
+    <t>44.468.700</t>
+  </si>
+  <si>
+    <t>PE08000346871</t>
+  </si>
+  <si>
+    <t>36.025.219</t>
+  </si>
+  <si>
+    <t>PE08000346847</t>
+  </si>
+  <si>
+    <t>11.023.839</t>
+  </si>
+  <si>
+    <t>PE08000346661</t>
+  </si>
+  <si>
+    <t>61.430.730</t>
+  </si>
+  <si>
+    <t>PE08000346555</t>
+  </si>
+  <si>
+    <t>13.736.883</t>
   </si>
 </sst>
 </file>
@@ -888,7 +1383,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -911,6 +1406,18 @@
     </font>
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -1060,12 +1567,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1440,58 +1959,52 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1503,74 +2016,80 @@
     <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1580,17 +2099,47 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2117,1255 +2666,3017 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B155"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15.75" outlineLevelCol="1"/>
+  <dimension ref="A1:J216"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="35.1428571428571" style="1" customWidth="1"/>
     <col min="2" max="2" width="25.4285714285714" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.14285714285714" style="1"/>
+    <col min="3" max="4" width="20.1428571428571" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.14285714285714" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" spans="1:2">
+    <row r="1" ht="16.5" spans="1:4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" ht="32.25" spans="1:2">
-      <c r="A2" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="48" spans="1:2">
-      <c r="A3" s="4" t="s">
+    <row r="2" spans="1:4">
+      <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" ht="48" spans="1:2">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D2" s="8">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" ht="32.25" spans="1:2">
-      <c r="A5" s="4" t="s">
+      <c r="B3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="D3" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="9" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" ht="32.25" spans="1:2">
-      <c r="A6" s="4" t="s">
+      <c r="B4" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="D4" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="9" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" ht="32.25" spans="1:2">
-      <c r="A7" s="4" t="s">
+      <c r="B5" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="D5" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" ht="48" spans="1:2">
-      <c r="A8" s="4" t="s">
+      <c r="B6" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="D6" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" ht="32.25" spans="1:2">
-      <c r="A9" s="4" t="s">
+      <c r="B7" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="D7" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" ht="32.25" spans="1:2">
-      <c r="A10" s="4" t="s">
+      <c r="B8" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="D8" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" ht="32.25" spans="1:2">
-      <c r="A11" s="4" t="s">
+      <c r="B9" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="D9" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" ht="32.25" spans="1:2">
-      <c r="A12" s="4" t="s">
+      <c r="B10" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="D10" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" ht="32.25" spans="1:2">
-      <c r="A13" s="4" t="s">
+      <c r="B11" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="D11" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" ht="32.25" spans="1:2">
-      <c r="A14" s="4" t="s">
+      <c r="B12" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="D12" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="9" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" ht="32.25" spans="1:2">
-      <c r="A15" s="4" t="s">
+      <c r="B13" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="D13" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="9" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" ht="32.25" spans="1:2">
-      <c r="A16" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="5" t="s">
+      <c r="B14" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="17" ht="32.25" spans="1:2">
-      <c r="A17" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="5" t="s">
+      <c r="D14" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="9" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="18" ht="32.25" spans="1:2">
-      <c r="A18" s="4" t="s">
+      <c r="B15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="D15" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="16" ht="30.75" spans="1:4">
+      <c r="A16" s="9" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="19" ht="32.25" spans="1:2">
-      <c r="A19" s="4" t="s">
+      <c r="B16" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="D16" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" ht="32.25" spans="1:2">
-      <c r="A20" s="4" t="s">
+    <row r="17" spans="1:4">
+      <c r="A17" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B17" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" ht="48" spans="1:2">
-      <c r="A21" s="4" t="s">
+      <c r="D17" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B18" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="22" ht="32.25" spans="1:2">
-      <c r="A22" s="4" t="s">
+      <c r="D18" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B19" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="23" ht="32.25" spans="1:2">
-      <c r="A23" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="5" t="s">
+      <c r="D19" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="9" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="24" ht="32.25" spans="1:2">
-      <c r="A24" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" s="5" t="s">
+      <c r="B20" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="25" ht="32.25" spans="1:2">
-      <c r="A25" s="4" t="s">
+      <c r="D20" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="21" ht="30.75" spans="1:4">
+      <c r="A21" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B21" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="26" ht="32.25" spans="1:2">
-      <c r="A26" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B26" s="5" t="s">
+      <c r="D21" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" ht="30.75" spans="1:4">
+      <c r="A22" s="9" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="27" ht="32.25" spans="1:2">
-      <c r="A27" s="4" t="s">
+      <c r="B22" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="D22" s="13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="28" ht="32.25" spans="1:2">
-      <c r="A28" s="4" t="s">
+    <row r="23" spans="1:4">
+      <c r="A23" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B23" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="29" ht="32.25" spans="1:2">
-      <c r="A29" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="5" t="s">
+      <c r="D23" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="24" ht="30.75" spans="1:4">
+      <c r="A24" s="9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="30" ht="32.25" spans="1:2">
-      <c r="A30" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B30" s="5" t="s">
+      <c r="B24" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" s="10" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="31" ht="32.25" spans="1:2">
-      <c r="A31" s="4" t="s">
+      <c r="D24" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B25" s="12" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="32" ht="32.25" spans="1:2">
-      <c r="A32" s="4" t="s">
+      <c r="C25" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="D25" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="9" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="33" ht="32.25" spans="1:2">
-      <c r="A33" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B33" s="5" t="s">
+      <c r="B26" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="34" ht="32.25" spans="1:2">
-      <c r="A34" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B34" s="5" t="s">
+      <c r="D26" s="14"/>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="35" ht="32.25" spans="1:2">
-      <c r="A35" s="4" t="s">
+      <c r="B27" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="D27" s="14"/>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="9" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="36" ht="32.25" spans="1:2">
-      <c r="A36" s="4" t="s">
+      <c r="B28" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="D28" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="9" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="37" ht="32.25" spans="1:2">
-      <c r="A37" s="4" t="s">
+      <c r="B29" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="D29" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="9" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="38" ht="32.25" spans="1:2">
-      <c r="A38" s="4" t="s">
+      <c r="B30" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="D30" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="9" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="39" ht="32.25" spans="1:2">
-      <c r="A39" s="4" t="s">
+      <c r="B31" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="D31" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="32" ht="30.75" spans="1:4">
+      <c r="A32" s="9" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="40" ht="32.25" spans="1:2">
-      <c r="A40" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B40" s="5" t="s">
+      <c r="B32" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" s="10" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="41" ht="32.25" spans="1:2">
-      <c r="A41" s="4" t="s">
+      <c r="D32" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="B41" s="5" t="s">
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="9" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="42" ht="32.25" spans="1:2">
-      <c r="A42" s="4" t="s">
+      <c r="B33" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="D33" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="34" ht="30.75" spans="1:4">
+      <c r="A34" s="9" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="43" ht="32.25" spans="1:2">
-      <c r="A43" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B43" s="5" t="s">
+      <c r="B34" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="44" ht="32.25" spans="1:2">
-      <c r="A44" s="4" t="s">
+      <c r="D34" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B35" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="10" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="45" ht="32.25" spans="1:2">
-      <c r="A45" s="4" t="s">
+      <c r="D35" s="14"/>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B36" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="10" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="46" ht="32.25" spans="1:2">
-      <c r="A46" s="4" t="s">
+      <c r="D36" s="14"/>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B37" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" s="10" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="47" ht="32.25" spans="1:2">
-      <c r="A47" s="4" t="s">
+      <c r="D37" s="14"/>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B38" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" s="10" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="48" ht="32.25" spans="1:2">
-      <c r="A48" s="4" t="s">
+      <c r="D38" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B39" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="49" ht="32.25" spans="1:2">
-      <c r="A49" s="4" t="s">
+      <c r="D39" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B40" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C40" s="10" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="50" ht="32.25" spans="1:2">
-      <c r="A50" s="4" t="s">
+      <c r="D40" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B41" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C41" s="10" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="51" ht="32.25" spans="1:2">
-      <c r="A51" s="4" t="s">
+      <c r="D41" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B42" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" s="10" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="52" ht="32.25" spans="1:2">
-      <c r="A52" s="4" t="s">
+      <c r="D42" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B43" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" s="10" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="53" ht="32.25" spans="1:2">
-      <c r="A53" s="4" t="s">
+      <c r="D43" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B44" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44" s="10" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="54" ht="32.25" spans="1:2">
-      <c r="A54" s="4" t="s">
+      <c r="D44" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="45" ht="30.75" spans="1:4">
+      <c r="A45" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B45" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" s="10" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="55" ht="32.25" spans="1:2">
-      <c r="A55" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B55" s="5" t="s">
+      <c r="D45" s="13" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="56" ht="32.25" spans="1:2">
-      <c r="A56" s="4" t="s">
+    <row r="46" spans="1:4">
+      <c r="A46" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B46" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46" s="10" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="57" ht="32.25" spans="1:2">
-      <c r="A57" s="4" t="s">
+      <c r="D46" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="B47" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" s="10" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="58" ht="32.25" spans="1:2">
-      <c r="A58" s="6" t="s">
+      <c r="D47" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B48" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="10" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="59" ht="32.25" spans="1:2">
-      <c r="A59" s="4" t="s">
+      <c r="D48" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="B49" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C49" s="10" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="60" ht="32.25" spans="1:2">
-      <c r="A60" s="4" t="s">
+      <c r="D49" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B50" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50" s="10" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="61" ht="32.25" spans="1:2">
-      <c r="A61" s="4" t="s">
+      <c r="D50" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="B51" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C51" s="10" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="62" ht="32.25" spans="1:2">
-      <c r="A62" s="4" t="s">
+      <c r="D51" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="52" ht="30.75" spans="1:4">
+      <c r="A52" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="B52" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C52" s="10" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="63" ht="32.25" spans="1:2">
-      <c r="A63" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B63" s="5" t="s">
+      <c r="D52" s="13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="9" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="64" ht="32.25" spans="1:2">
-      <c r="A64" s="4" t="s">
+      <c r="B53" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C53" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="D53" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="9" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="65" ht="32.25" spans="1:2">
-      <c r="A65" s="4" t="s">
+      <c r="B54" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C54" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="D54" s="14"/>
+    </row>
+    <row r="55" ht="30.75" spans="1:4">
+      <c r="A55" s="9" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="66" ht="32.25" spans="1:2">
-      <c r="A66" s="4" t="s">
+      <c r="B55" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C55" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="D55" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="9" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="67" ht="32.25" spans="1:2">
-      <c r="A67" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B67" s="5" t="s">
+      <c r="B56" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="68" ht="32.25" spans="1:2">
-      <c r="A68" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B68" s="5" t="s">
+      <c r="D56" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="9" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="69" ht="32.25" spans="1:2">
-      <c r="A69" s="4" t="s">
+      <c r="B57" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C57" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="D57" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="9" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="70" ht="32.25" spans="1:2">
-      <c r="A70" s="4" t="s">
+      <c r="B58" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="D58" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="9" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="71" ht="32.25" spans="1:2">
-      <c r="A71" s="4" t="s">
+      <c r="B59" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C59" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="D59" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="9" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="72" ht="32.25" spans="1:2">
-      <c r="A72" s="4" t="s">
+      <c r="B60" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C60" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B72" s="5" t="s">
+      <c r="D60" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="9" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="73" ht="32.25" spans="1:2">
-      <c r="A73" s="4" t="s">
+      <c r="B61" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C61" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B73" s="5" t="s">
+      <c r="D61" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="9" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="74" ht="32.25" spans="1:2">
-      <c r="A74" s="4" t="s">
+      <c r="B62" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B74" s="5" t="s">
+      <c r="D62" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="9" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="75" ht="32.25" spans="1:2">
-      <c r="A75" s="4" t="s">
+      <c r="B63" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C63" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B75" s="5" t="s">
+      <c r="D63" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="9" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="76" ht="32.25" spans="1:2">
-      <c r="A76" s="4" t="s">
+      <c r="B64" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C64" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B76" s="5" t="s">
+      <c r="D64" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="9" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="77" ht="32.25" spans="1:2">
-      <c r="A77" s="4" t="s">
+      <c r="B65" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="D65" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="9" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="78" ht="32.25" spans="1:2">
-      <c r="A78" s="4" t="s">
+      <c r="B66" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C66" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="D66" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="9" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="79" ht="32.25" spans="1:2">
-      <c r="A79" s="4" t="s">
+      <c r="B67" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C67" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="D67" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="9" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="80" ht="32.25" spans="1:2">
-      <c r="A80" s="4" t="s">
+      <c r="B68" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C68" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="D68" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="9" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="81" ht="32.25" spans="1:2">
-      <c r="A81" s="4" t="s">
+      <c r="B69" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C69" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="D69" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="9" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="82" ht="32.25" spans="1:2">
-      <c r="A82" s="4" t="s">
+      <c r="B70" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C70" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="B82" s="5" t="s">
+      <c r="D70" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="9" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="83" ht="32.25" spans="1:2">
-      <c r="A83" s="4" t="s">
+      <c r="B71" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C71" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="D71" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="9" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="84" ht="32.25" spans="1:2">
-      <c r="A84" s="4" t="s">
+      <c r="B72" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C72" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="B84" s="5" t="s">
+      <c r="D72" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="9" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="85" ht="32.25" spans="1:2">
-      <c r="A85" s="4" t="s">
+      <c r="B73" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C73" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="B85" s="5" t="s">
+      <c r="D73" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" s="9" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="86" ht="32.25" spans="1:2">
-      <c r="A86" s="4" t="s">
+      <c r="B74" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C74" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="B86" s="5" t="s">
+      <c r="D74" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75" s="9" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="87" ht="32.25" spans="1:2">
-      <c r="A87" s="4" t="s">
+      <c r="B75" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C75" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="D75" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76" s="9" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="88" ht="32.25" spans="1:2">
-      <c r="A88" s="4" t="s">
+      <c r="B76" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C76" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="D76" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77" s="9" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="89" ht="32.25" spans="1:2">
-      <c r="A89" s="4" t="s">
+      <c r="B77" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C77" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B89" s="5" t="s">
+      <c r="D77" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" s="9" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="90" ht="32.25" spans="1:2">
-      <c r="A90" s="4" t="s">
+      <c r="B78" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C78" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="B90" s="5" t="s">
+      <c r="D78" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" s="9" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="91" ht="32.25" spans="1:2">
-      <c r="A91" s="4" t="s">
+      <c r="B79" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C79" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="B91" s="5" t="s">
+      <c r="D79" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" s="9" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="92" ht="32.25" spans="1:2">
-      <c r="A92" s="4" t="s">
+      <c r="B80" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C80" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="B92" s="5" t="s">
+      <c r="D80" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81" s="9" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="93" ht="32.25" spans="1:2">
-      <c r="A93" s="4" t="s">
+      <c r="B81" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C81" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="B93" s="5" t="s">
+      <c r="D81" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
+      <c r="A82" s="9" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="94" ht="32.25" spans="1:2">
-      <c r="A94" s="4" t="s">
+      <c r="B82" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C82" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="B94" s="5" t="s">
+      <c r="D82" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83" s="9" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="95" ht="32.25" spans="1:2">
-      <c r="A95" s="4" t="s">
+      <c r="B83" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C83" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="B95" s="5" t="s">
+      <c r="D83" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
+      <c r="A84" s="9" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="96" ht="32.25" spans="1:2">
-      <c r="A96" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B96" s="5" t="s">
+      <c r="B84" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C84" s="10" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="97" ht="48" spans="1:2">
-      <c r="A97" s="4" t="s">
+      <c r="D84" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="B97" s="5" t="s">
+      <c r="B85" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C85" s="10" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="98" ht="32.25" spans="1:2">
-      <c r="A98" s="4" t="s">
+      <c r="D85" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="B98" s="5" t="s">
+      <c r="B86" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C86" s="10" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="99" ht="32.25" spans="1:2">
-      <c r="A99" s="4" t="s">
+      <c r="D86" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
+      <c r="A87" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B99" s="5" t="s">
+      <c r="B87" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87" s="10" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="100" ht="32.25" spans="1:2">
-      <c r="A100" s="4" t="s">
+      <c r="D87" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="B100" s="5" t="s">
+      <c r="B88" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C88" s="10" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="101" ht="48" spans="1:2">
-      <c r="A101" s="4" t="s">
+      <c r="D88" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
+      <c r="A89" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B101" s="5" t="s">
+      <c r="B89" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C89" s="10" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="102" ht="32.25" spans="1:2">
-      <c r="A102" s="4" t="s">
+      <c r="D89" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="B102" s="5" t="s">
+      <c r="B90" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" s="10" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="103" ht="32.25" spans="1:2">
-      <c r="A103" s="4" t="s">
+      <c r="D90" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
+      <c r="A91" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="B103" s="5" t="s">
+      <c r="B91" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C91" s="10" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="104" ht="32.25" spans="1:2">
-      <c r="A104" s="4" t="s">
+      <c r="D91" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="B104" s="5" t="s">
+      <c r="B92" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C92" s="10" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="105" ht="32.25" spans="1:2">
-      <c r="A105" s="4" t="s">
+      <c r="D92" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="B105" s="5" t="s">
+      <c r="B93" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C93" s="10" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="106" ht="32.25" spans="1:2">
-      <c r="A106" s="4" t="s">
+      <c r="D93" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="B106" s="5" t="s">
+      <c r="B94" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C94" s="10" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="107" ht="32.25" spans="1:2">
-      <c r="A107" s="4" t="s">
+      <c r="D94" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B107" s="5" t="s">
+      <c r="B95" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C95" s="10" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="108" ht="32.25" spans="1:2">
-      <c r="A108" s="4" t="s">
+      <c r="D95" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="B108" s="5" t="s">
+      <c r="B96" s="10" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="109" ht="32.25" spans="1:2">
-      <c r="A109" s="4" t="s">
+      <c r="C96" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="B109" s="5" t="s">
+      <c r="D96" s="14"/>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" s="9" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="110" ht="32.25" spans="1:2">
-      <c r="A110" s="4" t="s">
+      <c r="B97" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C97" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="B110" s="5" t="s">
+      <c r="D97" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
+      <c r="A98" s="9" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="111" ht="32.25" spans="1:2">
-      <c r="A111" s="4" t="s">
+      <c r="B98" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C98" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="B111" s="5" t="s">
+      <c r="D98" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="99" ht="30.75" spans="1:4">
+      <c r="A99" s="9" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="112" ht="32.25" spans="1:2">
-      <c r="A112" s="4" t="s">
+      <c r="B99" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C99" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="B112" s="5" t="s">
+      <c r="D99" s="13" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="113" ht="32.25" spans="1:2">
-      <c r="A113" s="4" t="s">
+    <row r="100" ht="30.75" spans="1:4">
+      <c r="A100" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B113" s="5" t="s">
+      <c r="B100" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C100" s="10" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="114" ht="32.25" spans="1:2">
-      <c r="A114" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B114" s="5" t="s">
+      <c r="D100" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
+      <c r="A101" s="9" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="115" ht="32.25" spans="1:2">
-      <c r="A115" s="4" t="s">
+      <c r="B101" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C101" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="B115" s="5" t="s">
+      <c r="D101" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4">
+      <c r="A102" s="9" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="116" ht="32.25" spans="1:2">
-      <c r="A116" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="B116" s="5" t="s">
+      <c r="B102" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C102" s="10" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="117" ht="32.25" spans="1:2">
-      <c r="A117" s="4" t="s">
+      <c r="D102" s="14"/>
+    </row>
+    <row r="103" spans="1:4">
+      <c r="A103" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="B117" s="5" t="s">
+      <c r="B103" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C103" s="10" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="118" ht="32.25" spans="1:2">
-      <c r="A118" s="4" t="s">
+      <c r="D103" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
+      <c r="A104" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="B118" s="5" t="s">
+      <c r="B104" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C104" s="10" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="119" ht="32.25" spans="1:2">
-      <c r="A119" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B119" s="5" t="s">
+      <c r="D104" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="105" ht="30.75" spans="1:4">
+      <c r="A105" s="9" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="120" ht="32.25" spans="1:2">
-      <c r="A120" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B120" s="5" t="s">
+      <c r="B105" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C105" s="10" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="121" ht="32.25" spans="1:2">
-      <c r="A121" s="4" t="s">
+      <c r="D105" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="B121" s="5" t="s">
+    </row>
+    <row r="106" ht="30.75" spans="1:4">
+      <c r="A106" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="122" ht="48" spans="1:2">
-      <c r="A122" s="4" t="s">
+      <c r="B106" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C106" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="B122" s="5" t="s">
+      <c r="D106" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="107" ht="30.75" spans="1:4">
+      <c r="A107" s="9" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="123" ht="32.25" spans="1:2">
-      <c r="A123" s="4" t="s">
+      <c r="B107" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C107" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="B123" s="5" t="s">
+      <c r="D107" s="13" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="124" ht="48" spans="1:2">
-      <c r="A124" s="4" t="s">
+    <row r="108" spans="1:4">
+      <c r="A108" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="B124" s="5" t="s">
+      <c r="B108" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C108" s="10" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="125" ht="48" spans="1:2">
-      <c r="A125" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="B125" s="5" t="s">
+      <c r="D108" s="14"/>
+    </row>
+    <row r="109" spans="1:4">
+      <c r="A109" s="9" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="126" ht="32.25" spans="1:2">
-      <c r="A126" s="4" t="s">
+      <c r="B109" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C109" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="B126" s="5" t="s">
+      <c r="D109" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="110" ht="30.75" spans="1:4">
+      <c r="A110" s="9" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="127" ht="32.25" spans="1:2">
-      <c r="A127" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="B127" s="5" t="s">
+      <c r="B110" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C110" s="10" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="128" ht="32.25" spans="1:2">
-      <c r="A128" s="4" t="s">
+      <c r="D110" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
+      <c r="A111" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B128" s="5" t="s">
+      <c r="B111" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C111" s="10" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="129" ht="32.25" spans="1:2">
-      <c r="A129" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="B129" s="5" t="s">
+      <c r="D111" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
+      <c r="A112" s="9" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="130" ht="32.25" spans="1:2">
-      <c r="A130" s="4" t="s">
+      <c r="B112" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C112" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="B130" s="5" t="s">
+      <c r="D112" s="14"/>
+    </row>
+    <row r="113" spans="1:4">
+      <c r="A113" s="9" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="131" ht="32.25" spans="1:2">
-      <c r="A131" s="4" t="s">
+      <c r="B113" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C113" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="B131" s="5" t="s">
+      <c r="D113" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="114" ht="30.75" spans="1:4">
+      <c r="A114" s="9" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="132" ht="32.25" spans="1:2">
-      <c r="A132" s="4" t="s">
+      <c r="B114" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C114" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="B132" s="5" t="s">
+      <c r="D114" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
+      <c r="A115" s="9" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="133" ht="32.25" spans="1:2">
-      <c r="A133" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="B133" s="5" t="s">
+      <c r="B115" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C115" s="10" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="134" ht="32.25" spans="1:2">
-      <c r="A134" s="4" t="s">
+      <c r="D115" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
+      <c r="A116" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="B134" s="5" t="s">
+      <c r="B116" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C116" s="10" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="135" ht="32.25" spans="1:2">
-      <c r="A135" s="4" t="s">
+      <c r="D116" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
+      <c r="A117" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="B135" s="5" t="s">
+      <c r="B117" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C117" s="10" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="136" ht="32.25" spans="1:2">
-      <c r="A136" s="4" t="s">
+      <c r="D117" s="14"/>
+    </row>
+    <row r="118" ht="30.75" spans="1:4">
+      <c r="A118" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="B136" s="5" t="s">
+      <c r="B118" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C118" s="10" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="137" ht="32.25" spans="1:2">
-      <c r="A137" s="4" t="s">
+      <c r="D118" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
+      <c r="A119" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="B137" s="5" t="s">
+      <c r="B119" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C119" s="10" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="138" ht="32.25" spans="1:2">
-      <c r="A138" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="B138" s="5" t="s">
+      <c r="D119" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4">
+      <c r="A120" s="9" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="139" ht="32.25" spans="1:2">
-      <c r="A139" s="4" t="s">
+      <c r="B120" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C120" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="B139" s="5" t="s">
+      <c r="D120" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
+      <c r="A121" s="9" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="140" ht="32.25" spans="1:2">
-      <c r="A140" s="4" t="s">
+      <c r="B121" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C121" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="B140" s="5" t="s">
+      <c r="D121" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="122" ht="30.75" spans="1:4">
+      <c r="A122" s="9" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="141" ht="32.25" spans="1:2">
-      <c r="A141" s="4" t="s">
+      <c r="B122" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C122" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="B141" s="5" t="s">
+      <c r="D122" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
+      <c r="A123" s="9" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="142" ht="32.25" spans="1:2">
-      <c r="A142" s="4" t="s">
+      <c r="B123" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C123" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="B142" s="5" t="s">
+      <c r="D123" s="14"/>
+    </row>
+    <row r="124" spans="1:4">
+      <c r="A124" s="9" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="143" ht="32.25" spans="1:2">
-      <c r="A143" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="B143" s="5" t="s">
+      <c r="B124" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C124" s="10" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="144" ht="32.25" spans="1:2">
-      <c r="A144" s="4" t="s">
+      <c r="D124" s="14"/>
+    </row>
+    <row r="125" spans="1:4">
+      <c r="A125" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="B144" s="5" t="s">
+      <c r="B125" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C125" s="10" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="145" ht="32.25" spans="1:2">
-      <c r="A145" s="4" t="s">
+      <c r="D125" s="14"/>
+    </row>
+    <row r="126" spans="1:4">
+      <c r="A126" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="B145" s="5" t="s">
+      <c r="B126" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C126" s="10" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="146" ht="32.25" spans="1:2">
-      <c r="A146" s="4" t="s">
+      <c r="D126" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4">
+      <c r="A127" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="B146" s="5" t="s">
+      <c r="B127" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C127" s="10" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="147" ht="32.25" spans="1:2">
-      <c r="A147" s="4" t="s">
+      <c r="D127" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
+      <c r="A128" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="B147" s="5" t="s">
+      <c r="B128" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C128" s="10" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="148" ht="32.25" spans="1:2">
-      <c r="A148" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="B148" s="5" t="s">
+      <c r="D128" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4">
+      <c r="A129" s="9" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="149" ht="32.25" spans="1:2">
-      <c r="A149" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="B149" s="5" t="s">
+      <c r="B129" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C129" s="10" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="150" ht="32.25" spans="1:2">
-      <c r="A150" s="4" t="s">
+      <c r="D129" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4">
+      <c r="A130" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="B150" s="5" t="s">
+      <c r="B130" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C130" s="10" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="151" ht="32.25" spans="1:2">
-      <c r="A151" s="4" t="s">
+      <c r="D130" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
+      <c r="A131" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="B151" s="5" t="s">
+      <c r="B131" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C131" s="10" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="152" ht="32.25" spans="1:2">
-      <c r="A152" s="4" t="s">
+      <c r="D131" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
+      <c r="A132" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B152" s="5" t="s">
+      <c r="B132" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C132" s="10" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="153" ht="32.25" spans="1:2">
-      <c r="A153" s="4" t="s">
+      <c r="D132" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
+      <c r="A133" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="B153" s="5" t="s">
+      <c r="B133" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C133" s="10" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="154" ht="32.25" spans="1:2">
-      <c r="A154" s="4" t="s">
+      <c r="D133" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
+      <c r="A134" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="B154" s="5" t="s">
+      <c r="B134" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C134" s="10" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="155" ht="32.25" spans="1:2">
-      <c r="A155" s="4" t="s">
+      <c r="D134" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="B155" s="5" t="s">
+      <c r="B135" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C135" s="10" t="s">
         <v>282</v>
       </c>
+      <c r="D135" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="B136" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C136" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="D136" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="B137" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C137" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="D137" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4">
+      <c r="A138" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="B138" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C138" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="D138" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="B139" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C139" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="D139" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="B140" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C140" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="D140" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="B141" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C141" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="D141" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4">
+      <c r="A142" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="B142" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C142" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="D142" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4">
+      <c r="A143" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="B143" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C143" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="D143" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4">
+      <c r="A144" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="B144" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C144" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="D144" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5">
+      <c r="A145" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="B145" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C145" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="D145" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5">
+      <c r="A146" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="B146" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C146" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="D146" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5">
+      <c r="A147" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="B147" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C147" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="D147" s="14"/>
+    </row>
+    <row r="148" spans="1:5">
+      <c r="A148" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="B148" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C148" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="D148" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5">
+      <c r="A149" s="9" t="s">
+        <v>309</v>
+      </c>
+      <c r="B149" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C149" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="D149" s="14"/>
+    </row>
+    <row r="150" spans="1:5">
+      <c r="A150" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="B150" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C150" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="D150" s="14"/>
+    </row>
+    <row r="151" spans="1:5">
+      <c r="A151" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="B151" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C151" s="10" t="s">
+        <v>314</v>
+      </c>
+      <c r="D151" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="152" ht="16.5" spans="1:5">
+      <c r="A152" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="B152" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C152" s="10" t="s">
+        <v>316</v>
+      </c>
+      <c r="D152" s="14"/>
+      <c r="E152" s="16"/>
+    </row>
+    <row r="153" ht="16.5" spans="1:5">
+      <c r="A153" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="B153" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C153" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="D153" s="11">
+        <v>46177</v>
+      </c>
+      <c r="E153" s="16"/>
+    </row>
+    <row r="154" ht="16.5" spans="1:5">
+      <c r="A154" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="B154" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C154" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="D154" s="14"/>
+      <c r="E154" s="16"/>
+    </row>
+    <row r="155" ht="16.5" spans="1:5">
+      <c r="A155" s="9" t="s">
+        <v>321</v>
+      </c>
+      <c r="B155" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C155" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="D155" s="11">
+        <v>46177</v>
+      </c>
+      <c r="E155" s="16"/>
+    </row>
+    <row r="156" ht="16.5" spans="1:5">
+      <c r="A156" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="B156" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C156" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="D156" s="11">
+        <v>46238</v>
+      </c>
+      <c r="E156" s="16"/>
+    </row>
+    <row r="157" ht="16.5" spans="1:5">
+      <c r="A157" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="B157" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C157" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="D157" s="14"/>
+      <c r="E157" s="16"/>
+    </row>
+    <row r="158" ht="30.75" spans="1:5">
+      <c r="A158" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="B158" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C158" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="D158" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E158" s="16"/>
+    </row>
+    <row r="159" ht="30.75" spans="1:5">
+      <c r="A159" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="B159" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C159" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="D159" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E159" s="16"/>
+    </row>
+    <row r="160" ht="30.75" spans="1:5">
+      <c r="A160" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="B160" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C160" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="D160" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E160" s="16"/>
+    </row>
+    <row r="161" ht="16.5" spans="1:10">
+      <c r="A161" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="B161" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C161" s="10" t="s">
+        <v>336</v>
+      </c>
+      <c r="D161" s="11">
+        <v>46207</v>
+      </c>
+      <c r="E161" s="16"/>
+    </row>
+    <row r="162" ht="30.75" spans="1:10">
+      <c r="A162" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="B162" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C162" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="D162" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="E162" s="16"/>
+    </row>
+    <row r="163" ht="30.75" spans="1:10">
+      <c r="A163" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="B163" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C163" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="D163" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E163" s="16"/>
+    </row>
+    <row r="164" ht="30.75" spans="1:10">
+      <c r="A164" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="B164" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C164" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="D164" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E164" s="16"/>
+      <c r="J164" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="165" ht="16.5" spans="1:10">
+      <c r="A165" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="B165" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C165" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="D165" s="11">
+        <v>46146</v>
+      </c>
+      <c r="E165" s="16"/>
+    </row>
+    <row r="166" ht="16.5" spans="1:10">
+      <c r="A166" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="B166" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C166" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="D166" s="11">
+        <v>46146</v>
+      </c>
+      <c r="E166" s="16"/>
+    </row>
+    <row r="167" ht="30.75" spans="1:10">
+      <c r="A167" s="9" t="s">
+        <v>347</v>
+      </c>
+      <c r="B167" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C167" s="10" t="s">
+        <v>348</v>
+      </c>
+      <c r="D167" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E167" s="16"/>
+    </row>
+    <row r="168" ht="30.75" spans="1:10">
+      <c r="A168" s="9" t="s">
+        <v>349</v>
+      </c>
+      <c r="B168" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C168" s="10" t="s">
+        <v>350</v>
+      </c>
+      <c r="D168" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E168" s="16"/>
+    </row>
+    <row r="169" ht="30.75" spans="1:10">
+      <c r="A169" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="B169" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C169" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="D169" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E169" s="16"/>
+    </row>
+    <row r="170" ht="30.75" spans="1:10">
+      <c r="A170" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="B170" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C170" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="D170" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E170" s="16"/>
+    </row>
+    <row r="171" ht="30.75" spans="1:10">
+      <c r="A171" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="B171" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C171" s="10" t="s">
+        <v>356</v>
+      </c>
+      <c r="D171" s="13" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="172" ht="30.75" spans="1:10">
+      <c r="A172" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="B172" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C172" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="D172" s="13" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10">
+      <c r="A173" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="B173" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C173" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="D173" s="14"/>
+    </row>
+    <row r="174" spans="1:10">
+      <c r="A174" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="B174" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="C174" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D174" s="14"/>
+    </row>
+    <row r="175" spans="1:10">
+      <c r="A175" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="B175" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C175" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="D175" s="14"/>
+    </row>
+    <row r="176" spans="1:10">
+      <c r="A176" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B176" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C176" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="D176" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4">
+      <c r="A177" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="B177" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C177" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="D177" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4">
+      <c r="A178" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="B178" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C178" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="D178" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4">
+      <c r="A179" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="B179" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C179" s="10" t="s">
+        <v>372</v>
+      </c>
+      <c r="D179" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4">
+      <c r="A180" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="B180" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C180" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="D180" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4">
+      <c r="A181" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="B181" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C181" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="D181" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4">
+      <c r="A182" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="B182" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C182" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="D182" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4">
+      <c r="A183" s="9" t="s">
+        <v>379</v>
+      </c>
+      <c r="B183" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C183" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="D183" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4">
+      <c r="A184" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="B184" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C184" s="10" t="s">
+        <v>382</v>
+      </c>
+      <c r="D184" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4">
+      <c r="A185" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="B185" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C185" s="10" t="s">
+        <v>384</v>
+      </c>
+      <c r="D185" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4">
+      <c r="A186" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="B186" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C186" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="D186" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4">
+      <c r="A187" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="B187" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C187" s="10" t="s">
+        <v>388</v>
+      </c>
+      <c r="D187" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4">
+      <c r="A188" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="B188" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C188" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="D188" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4">
+      <c r="A189" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="B189" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C189" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="D189" s="14"/>
+    </row>
+    <row r="190" ht="30.75" spans="1:4">
+      <c r="A190" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="B190" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C190" s="10" t="s">
+        <v>394</v>
+      </c>
+      <c r="D190" s="13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4">
+      <c r="A191" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="B191" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C191" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="D191" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="192" ht="30.75" spans="1:4">
+      <c r="A192" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="B192" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C192" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="D192" s="13" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4">
+      <c r="A193" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="B193" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C193" s="10" t="s">
+        <v>401</v>
+      </c>
+      <c r="D193" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4">
+      <c r="A194" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="B194" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C194" s="10" t="s">
+        <v>403</v>
+      </c>
+      <c r="D194" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4">
+      <c r="A195" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="B195" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C195" s="10" t="s">
+        <v>405</v>
+      </c>
+      <c r="D195" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4">
+      <c r="A196" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="B196" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C196" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="D196" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4">
+      <c r="A197" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="B197" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C197" s="10" t="s">
+        <v>409</v>
+      </c>
+      <c r="D197" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4">
+      <c r="A198" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="B198" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C198" s="10" t="s">
+        <v>411</v>
+      </c>
+      <c r="D198" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4">
+      <c r="A199" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="B199" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C199" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="D199" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4">
+      <c r="A200" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="B200" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C200" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="D200" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4">
+      <c r="A201" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="B201" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C201" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="D201" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="202" ht="30.75" spans="1:4">
+      <c r="A202" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="B202" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C202" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D202" s="13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4">
+      <c r="A203" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="B203" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C203" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="D203" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4">
+      <c r="A204" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="B204" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C204" s="10">
+        <v>329.227</v>
+      </c>
+      <c r="D204" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4">
+      <c r="A205" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="B205" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C205" s="10" t="s">
+        <v>424</v>
+      </c>
+      <c r="D205" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="206" ht="30.75" spans="1:4">
+      <c r="A206" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="B206" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C206" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="D206" s="13" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4">
+      <c r="A207" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="B207" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C207" s="10" t="s">
+        <v>428</v>
+      </c>
+      <c r="D207" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4">
+      <c r="A208" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="B208" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C208" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="D208" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4">
+      <c r="A209" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="B209" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C209" s="10" t="s">
+        <v>432</v>
+      </c>
+      <c r="D209" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4">
+      <c r="A210" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="B210" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C210" s="10" t="s">
+        <v>434</v>
+      </c>
+      <c r="D210" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4">
+      <c r="A211" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="B211" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C211" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="D211" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4">
+      <c r="A212" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="B212" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C212" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="D212" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4">
+      <c r="A213" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="B213" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C213" s="10" t="s">
+        <v>440</v>
+      </c>
+      <c r="D213" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4">
+      <c r="A214" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="B214" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C214" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="D214" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4">
+      <c r="A215" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="B215" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C215" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="D215" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4">
+      <c r="A216" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="B216" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C216" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D216" s="11">
+        <v>46146</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:E151" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
chore(deploy): prod compose image name, .env-only flow, docker seed script, SCP deploy doc; remove .env.prod.example
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/maHĐ.xlsx
+++ b/maHĐ.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$151</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -27,14 +30,29 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="447">
   <si>
     <t>MÃ KHÁCH HÀNG</t>
   </si>
   <si>
+    <t>EVN</t>
+  </si>
+  <si>
     <t>SỐ TIỀN</t>
   </si>
   <si>
+    <t>HẠN THANH TOÁN</t>
+  </si>
+  <si>
+    <t>PC03PP0243527</t>
+  </si>
+  <si>
+    <t>EVNCPC</t>
+  </si>
+  <si>
+    <t>80.751.276</t>
+  </si>
+  <si>
     <t>PC03GG0718405</t>
   </si>
   <si>
@@ -119,10 +137,7 @@
     <t>11.254.384</t>
   </si>
   <si>
-    <t>8.360.029</t>
-  </si>
-  <si>
-    <t>12.157.893</t>
+    <t>17/03/2026</t>
   </si>
   <si>
     <t>PC08BB0252277</t>
@@ -155,19 +170,13 @@
     <t>18.624.481</t>
   </si>
   <si>
-    <t>16.442.603</t>
-  </si>
-  <si>
-    <t>16.464.699</t>
-  </si>
-  <si>
     <t>PC03DD0479701</t>
   </si>
   <si>
     <t>53.589.442</t>
   </si>
   <si>
-    <t>56.474.021</t>
+    <t>23/03/2026</t>
   </si>
   <si>
     <t>PC08FF0619324</t>
@@ -182,21 +191,21 @@
     <t>55.393.928</t>
   </si>
   <si>
-    <t>45.219.172</t>
-  </si>
-  <si>
-    <t>54.421.040</t>
-  </si>
-  <si>
     <t>PD27007696347</t>
   </si>
   <si>
+    <t>EVNHANOI</t>
+  </si>
+  <si>
     <t>239.728.637</t>
   </si>
   <si>
     <t>PA22040530046</t>
   </si>
   <si>
+    <t>EVNNCP</t>
+  </si>
+  <si>
     <t>99.625.896</t>
   </si>
   <si>
@@ -206,9 +215,6 @@
     <t>10.795.162</t>
   </si>
   <si>
-    <t>13.991.875</t>
-  </si>
-  <si>
     <t>PA25VT0039197</t>
   </si>
   <si>
@@ -239,7 +245,7 @@
     <t>125.086.291</t>
   </si>
   <si>
-    <t>131.207.558</t>
+    <t>22/03/2026</t>
   </si>
   <si>
     <t>PA02PT0024884</t>
@@ -254,9 +260,6 @@
     <t>94.018.061</t>
   </si>
   <si>
-    <t>104.195.462</t>
-  </si>
-  <si>
     <t>PA25BX0025561</t>
   </si>
   <si>
@@ -323,7 +326,7 @@
     <t>77.948.158</t>
   </si>
   <si>
-    <t>103.157.911</t>
+    <t>20/03/2026</t>
   </si>
   <si>
     <t>PNTD003012612</t>
@@ -368,9 +371,6 @@
     <t>63.630.440</t>
   </si>
   <si>
-    <t>71.899.015</t>
-  </si>
-  <si>
     <t>PC02DD0552944</t>
   </si>
   <si>
@@ -389,12 +389,6 @@
     <t>4.514.078</t>
   </si>
   <si>
-    <t>2.808.287</t>
-  </si>
-  <si>
-    <t>4.759.039</t>
-  </si>
-  <si>
     <t>PC01EE0573816</t>
   </si>
   <si>
@@ -557,9 +551,6 @@
     <t>20.405.084</t>
   </si>
   <si>
-    <t>65.658.440</t>
-  </si>
-  <si>
     <t>PC02KK0924548</t>
   </si>
   <si>
@@ -641,6 +632,9 @@
     <t>PB16060029755</t>
   </si>
   <si>
+    <t>EVNSPC</t>
+  </si>
+  <si>
     <t>4.837.085</t>
   </si>
   <si>
@@ -662,7 +656,7 @@
     <t>141.697.728</t>
   </si>
   <si>
-    <t>308.785.427</t>
+    <t>19/03/2026</t>
   </si>
   <si>
     <t>PA04TP1480282</t>
@@ -671,27 +665,12 @@
     <t>87.951.744</t>
   </si>
   <si>
-    <t>105.165.475</t>
-  </si>
-  <si>
     <t>PA18LC0108438</t>
   </si>
   <si>
     <t>116.694.432</t>
   </si>
   <si>
-    <t>PNNB000047048</t>
-  </si>
-  <si>
-    <t>316.974.643</t>
-  </si>
-  <si>
-    <t>199.974.643</t>
-  </si>
-  <si>
-    <t>342.588.604</t>
-  </si>
-  <si>
     <t>PA11CL0030910</t>
   </si>
   <si>
@@ -716,7 +695,7 @@
     <t>79.292.736</t>
   </si>
   <si>
-    <t>79.320.038</t>
+    <t>24/03/2026</t>
   </si>
   <si>
     <t>PM01009091017</t>
@@ -725,16 +704,13 @@
     <t>68.788.570</t>
   </si>
   <si>
-    <t>85.945.795</t>
-  </si>
-  <si>
     <t>PM13000373400</t>
   </si>
   <si>
     <t>169.010.323</t>
   </si>
   <si>
-    <t>188.830.310</t>
+    <t>21/03/2026</t>
   </si>
   <si>
     <t>PA05090091270</t>
@@ -755,9 +731,6 @@
     <t>78.624.756</t>
   </si>
   <si>
-    <t>79.512.732</t>
-  </si>
-  <si>
     <t>PA17LS0033396</t>
   </si>
   <si>
@@ -782,9 +755,6 @@
     <t>151.670.448</t>
   </si>
   <si>
-    <t>172.592.424</t>
-  </si>
-  <si>
     <t>PM21000062233</t>
   </si>
   <si>
@@ -809,9 +779,6 @@
     <t>105.721.718</t>
   </si>
   <si>
-    <t>119.741.818</t>
-  </si>
-  <si>
     <t>PA18VB0028340</t>
   </si>
   <si>
@@ -836,12 +803,6 @@
     <t>17.921.088</t>
   </si>
   <si>
-    <t>12.329.626</t>
-  </si>
-  <si>
-    <t>14.354.150</t>
-  </si>
-  <si>
     <t>PA02DH1026489</t>
   </si>
   <si>
@@ -876,6 +837,540 @@
   </si>
   <si>
     <t>64.376.208</t>
+  </si>
+  <si>
+    <t>PA02YL0029500</t>
+  </si>
+  <si>
+    <t>92.848.872</t>
+  </si>
+  <si>
+    <t>PA02TN0034159</t>
+  </si>
+  <si>
+    <t>104.010.048</t>
+  </si>
+  <si>
+    <t>PA02TN0034414</t>
+  </si>
+  <si>
+    <t>45.130.694</t>
+  </si>
+  <si>
+    <t>PA02TT0041868</t>
+  </si>
+  <si>
+    <t>126.433.267</t>
+  </si>
+  <si>
+    <t>PA02TT0044820</t>
+  </si>
+  <si>
+    <t>140.470.157</t>
+  </si>
+  <si>
+    <t>PA02LT0016984</t>
+  </si>
+  <si>
+    <t>160.788.672</t>
+  </si>
+  <si>
+    <t>PA02LT0017753</t>
+  </si>
+  <si>
+    <t>85.598.986</t>
+  </si>
+  <si>
+    <t>PA02LT0017786</t>
+  </si>
+  <si>
+    <t>88.349.184</t>
+  </si>
+  <si>
+    <t>PA02HH0036488</t>
+  </si>
+  <si>
+    <t>34.197.811</t>
+  </si>
+  <si>
+    <t>PA02HH0040202</t>
+  </si>
+  <si>
+    <t>27.846.374</t>
+  </si>
+  <si>
+    <t>PA02HH0042655</t>
+  </si>
+  <si>
+    <t>10.809.504</t>
+  </si>
+  <si>
+    <t>PA02HH0043104</t>
+  </si>
+  <si>
+    <t>25.997.760</t>
+  </si>
+  <si>
+    <t>PA02HH0043143</t>
+  </si>
+  <si>
+    <t>145.769.976</t>
+  </si>
+  <si>
+    <t>PA29020025651</t>
+  </si>
+  <si>
+    <t>86.805.043</t>
+  </si>
+  <si>
+    <t>PA29010022064</t>
+  </si>
+  <si>
+    <t>37.572.077</t>
+  </si>
+  <si>
+    <t>PA29010022062</t>
+  </si>
+  <si>
+    <t>20.047.565</t>
+  </si>
+  <si>
+    <t>PA29010022063</t>
+  </si>
+  <si>
+    <t>42.603.494</t>
+  </si>
+  <si>
+    <t>PA29010021429</t>
+  </si>
+  <si>
+    <t>26.916.138</t>
+  </si>
+  <si>
+    <t>PA10020328445</t>
+  </si>
+  <si>
+    <t>83.873.750</t>
+  </si>
+  <si>
+    <t>PA10020329686</t>
+  </si>
+  <si>
+    <t>26.556.595</t>
+  </si>
+  <si>
+    <t>PA10020329905</t>
+  </si>
+  <si>
+    <t>133.479.891</t>
+  </si>
+  <si>
+    <t>PB11020077036</t>
+  </si>
+  <si>
+    <t>138.051.065</t>
+  </si>
+  <si>
+    <t>PB11070059740</t>
+  </si>
+  <si>
+    <t>36.817.680</t>
+  </si>
+  <si>
+    <t>PB11020077039</t>
+  </si>
+  <si>
+    <t>74.046.882</t>
+  </si>
+  <si>
+    <t>PB09020086057</t>
+  </si>
+  <si>
+    <t>109.101.205</t>
+  </si>
+  <si>
+    <t>PNKS000136665</t>
+  </si>
+  <si>
+    <t>186.947.775</t>
+  </si>
+  <si>
+    <t>PE10000278727</t>
+  </si>
+  <si>
+    <t>EVNHCM</t>
+  </si>
+  <si>
+    <t>15.142.254</t>
+  </si>
+  <si>
+    <t>PK07000199578</t>
+  </si>
+  <si>
+    <t>7.552.373</t>
+  </si>
+  <si>
+    <t>PE01000134913</t>
+  </si>
+  <si>
+    <t>148.257.253</t>
+  </si>
+  <si>
+    <t>PP08000957588</t>
+  </si>
+  <si>
+    <t>53.595.808</t>
+  </si>
+  <si>
+    <t>15/03/2026</t>
+  </si>
+  <si>
+    <t>PP08000957769</t>
+  </si>
+  <si>
+    <t>59.792.729</t>
+  </si>
+  <si>
+    <t>PA25VY0071755</t>
+  </si>
+  <si>
+    <t>115.717.594</t>
+  </si>
+  <si>
+    <t>PA25TM0048571</t>
+  </si>
+  <si>
+    <t>107.440.819</t>
+  </si>
+  <si>
+    <t>PNYK000052011</t>
+  </si>
+  <si>
+    <t>85.721.544</t>
+  </si>
+  <si>
+    <t>PC03CC0030584</t>
+  </si>
+  <si>
+    <t>14.320.662</t>
+  </si>
+  <si>
+    <t>PC03BB0252696</t>
+  </si>
+  <si>
+    <t>120.128.486</t>
+  </si>
+  <si>
+    <t>PB09010084064</t>
+  </si>
+  <si>
+    <t>80.764.111</t>
+  </si>
+  <si>
+    <t>PB09010084065</t>
+  </si>
+  <si>
+    <t>90.546.373</t>
+  </si>
+  <si>
+    <t>PB14040069969</t>
+  </si>
+  <si>
+    <t>20.209.232</t>
+  </si>
+  <si>
+    <t>PB14040071353</t>
+  </si>
+  <si>
+    <t>74.977.667</t>
+  </si>
+  <si>
+    <t>PB06030117011</t>
+  </si>
+  <si>
+    <t>22.888.254</t>
+  </si>
+  <si>
+    <t>PB06030117044</t>
+  </si>
+  <si>
+    <t>43.914.658</t>
+  </si>
+  <si>
+    <t>PB06030117047</t>
+  </si>
+  <si>
+    <t>26.723.153</t>
+  </si>
+  <si>
+    <t>PB06030118340</t>
+  </si>
+  <si>
+    <t>112.415.979</t>
+  </si>
+  <si>
+    <t>PE16000375479</t>
+  </si>
+  <si>
+    <t>99.326.062</t>
+  </si>
+  <si>
+    <t>PE16000376253</t>
+  </si>
+  <si>
+    <t>101.883.032</t>
+  </si>
+  <si>
+    <t>PA09010245489</t>
+  </si>
+  <si>
+    <t>46.487.032</t>
+  </si>
+  <si>
+    <t>PB05060063421</t>
+  </si>
+  <si>
+    <t>51.333.517</t>
+  </si>
+  <si>
+    <t>PQ11000529289</t>
+  </si>
+  <si>
+    <t>11.128.320</t>
+  </si>
+  <si>
+    <t>PQ11000529196</t>
+  </si>
+  <si>
+    <t>48.428.833</t>
+  </si>
+  <si>
+    <t>PQ06000626200</t>
+  </si>
+  <si>
+    <t>45.253.356</t>
+  </si>
+  <si>
+    <t>PP03000966767</t>
+  </si>
+  <si>
+    <t>1.554.206</t>
+  </si>
+  <si>
+    <t>PNNQ003532279</t>
+  </si>
+  <si>
+    <t>60.601.383</t>
+  </si>
+  <si>
+    <t>PNNQ003532150</t>
+  </si>
+  <si>
+    <t>66.588.534</t>
+  </si>
+  <si>
+    <t>PNNQ003531890</t>
+  </si>
+  <si>
+    <t>143.579.254</t>
+  </si>
+  <si>
+    <t>PM23000092476</t>
+  </si>
+  <si>
+    <t>132.036.912</t>
+  </si>
+  <si>
+    <t>PM21000061960</t>
+  </si>
+  <si>
+    <t>113.836.579</t>
+  </si>
+  <si>
+    <t>PM21000061284</t>
+  </si>
+  <si>
+    <t>107.761.402</t>
+  </si>
+  <si>
+    <t>PM19000016004</t>
+  </si>
+  <si>
+    <t>124.604.179</t>
+  </si>
+  <si>
+    <t>PM17000099894</t>
+  </si>
+  <si>
+    <t>108.732.326</t>
+  </si>
+  <si>
+    <t>PM07000055838</t>
+  </si>
+  <si>
+    <t>137.550.744</t>
+  </si>
+  <si>
+    <t>PM05000019758</t>
+  </si>
+  <si>
+    <t>49.904.294</t>
+  </si>
+  <si>
+    <t>PM03000069761</t>
+  </si>
+  <si>
+    <t>101.034.734</t>
+  </si>
+  <si>
+    <t>PH14000006785</t>
+  </si>
+  <si>
+    <t>62.377.344</t>
+  </si>
+  <si>
+    <t>16/03/2026</t>
+  </si>
+  <si>
+    <t>PH11000731714</t>
+  </si>
+  <si>
+    <t>210.458.736</t>
+  </si>
+  <si>
+    <t>PH11000731682</t>
+  </si>
+  <si>
+    <t>25.766.554</t>
+  </si>
+  <si>
+    <t>PH10000023640</t>
+  </si>
+  <si>
+    <t>107.774.842</t>
+  </si>
+  <si>
+    <t>PH09000049549</t>
+  </si>
+  <si>
+    <t>57.558.470</t>
+  </si>
+  <si>
+    <t>PH04000073400</t>
+  </si>
+  <si>
+    <t>32.410.195</t>
+  </si>
+  <si>
+    <t>PE15000404717</t>
+  </si>
+  <si>
+    <t>132.410.637</t>
+  </si>
+  <si>
+    <t>PE15000403394</t>
+  </si>
+  <si>
+    <t>19.379.650</t>
+  </si>
+  <si>
+    <t>PE15000403346</t>
+  </si>
+  <si>
+    <t>45.081.092</t>
+  </si>
+  <si>
+    <t>PE15000403226</t>
+  </si>
+  <si>
+    <t>36.717.149</t>
+  </si>
+  <si>
+    <t>PE11002070284</t>
+  </si>
+  <si>
+    <t>55.378.817</t>
+  </si>
+  <si>
+    <t>PE11002069978</t>
+  </si>
+  <si>
+    <t>84.546.236</t>
+  </si>
+  <si>
+    <t>PE10000277229</t>
+  </si>
+  <si>
+    <t>PE10000276176</t>
+  </si>
+  <si>
+    <t>225.678.614</t>
+  </si>
+  <si>
+    <t>PE10000275961</t>
+  </si>
+  <si>
+    <t>150.597.516</t>
+  </si>
+  <si>
+    <t>PE10000275713</t>
+  </si>
+  <si>
+    <t>147.347.813</t>
+  </si>
+  <si>
+    <t>PE10000273214</t>
+  </si>
+  <si>
+    <t>101.792.484</t>
+  </si>
+  <si>
+    <t>PE10000270053</t>
+  </si>
+  <si>
+    <t>131.006.786</t>
+  </si>
+  <si>
+    <t>PE10000269648</t>
+  </si>
+  <si>
+    <t>61.326.677</t>
+  </si>
+  <si>
+    <t>PE08000347173</t>
+  </si>
+  <si>
+    <t>175.684.339</t>
+  </si>
+  <si>
+    <t>PE08000347113</t>
+  </si>
+  <si>
+    <t>44.468.700</t>
+  </si>
+  <si>
+    <t>PE08000346871</t>
+  </si>
+  <si>
+    <t>36.025.219</t>
+  </si>
+  <si>
+    <t>PE08000346847</t>
+  </si>
+  <si>
+    <t>11.023.839</t>
+  </si>
+  <si>
+    <t>PE08000346661</t>
+  </si>
+  <si>
+    <t>61.430.730</t>
+  </si>
+  <si>
+    <t>PE08000346555</t>
+  </si>
+  <si>
+    <t>13.736.883</t>
   </si>
 </sst>
 </file>
@@ -888,7 +1383,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -911,6 +1406,18 @@
     </font>
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -1060,12 +1567,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1440,58 +1959,52 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1503,74 +2016,80 @@
     <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1580,17 +2099,47 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2117,1255 +2666,3017 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B155"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15.75" outlineLevelCol="1"/>
+  <dimension ref="A1:J216"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="35.1428571428571" style="1" customWidth="1"/>
     <col min="2" max="2" width="25.4285714285714" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.14285714285714" style="1"/>
+    <col min="3" max="4" width="20.1428571428571" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.14285714285714" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" spans="1:2">
+    <row r="1" ht="16.5" spans="1:4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" ht="32.25" spans="1:2">
-      <c r="A2" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="48" spans="1:2">
-      <c r="A3" s="4" t="s">
+    <row r="2" spans="1:4">
+      <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" ht="48" spans="1:2">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D2" s="8">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" ht="32.25" spans="1:2">
-      <c r="A5" s="4" t="s">
+      <c r="B3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="D3" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="9" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" ht="32.25" spans="1:2">
-      <c r="A6" s="4" t="s">
+      <c r="B4" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="D4" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="9" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" ht="32.25" spans="1:2">
-      <c r="A7" s="4" t="s">
+      <c r="B5" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="D5" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" ht="48" spans="1:2">
-      <c r="A8" s="4" t="s">
+      <c r="B6" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="D6" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" ht="32.25" spans="1:2">
-      <c r="A9" s="4" t="s">
+      <c r="B7" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="D7" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" ht="32.25" spans="1:2">
-      <c r="A10" s="4" t="s">
+      <c r="B8" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="D8" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" ht="32.25" spans="1:2">
-      <c r="A11" s="4" t="s">
+      <c r="B9" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="D9" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" ht="32.25" spans="1:2">
-      <c r="A12" s="4" t="s">
+      <c r="B10" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="D10" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" ht="32.25" spans="1:2">
-      <c r="A13" s="4" t="s">
+      <c r="B11" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="D11" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" ht="32.25" spans="1:2">
-      <c r="A14" s="4" t="s">
+      <c r="B12" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="D12" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="9" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" ht="32.25" spans="1:2">
-      <c r="A15" s="4" t="s">
+      <c r="B13" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="D13" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="9" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" ht="32.25" spans="1:2">
-      <c r="A16" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="5" t="s">
+      <c r="B14" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="17" ht="32.25" spans="1:2">
-      <c r="A17" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="5" t="s">
+      <c r="D14" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="9" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="18" ht="32.25" spans="1:2">
-      <c r="A18" s="4" t="s">
+      <c r="B15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="D15" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="16" ht="30.75" spans="1:4">
+      <c r="A16" s="9" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="19" ht="32.25" spans="1:2">
-      <c r="A19" s="4" t="s">
+      <c r="B16" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="D16" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" ht="32.25" spans="1:2">
-      <c r="A20" s="4" t="s">
+    <row r="17" spans="1:4">
+      <c r="A17" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B17" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" ht="48" spans="1:2">
-      <c r="A21" s="4" t="s">
+      <c r="D17" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B18" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="22" ht="32.25" spans="1:2">
-      <c r="A22" s="4" t="s">
+      <c r="D18" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B19" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="23" ht="32.25" spans="1:2">
-      <c r="A23" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="5" t="s">
+      <c r="D19" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="9" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="24" ht="32.25" spans="1:2">
-      <c r="A24" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" s="5" t="s">
+      <c r="B20" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="25" ht="32.25" spans="1:2">
-      <c r="A25" s="4" t="s">
+      <c r="D20" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="21" ht="30.75" spans="1:4">
+      <c r="A21" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B21" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="26" ht="32.25" spans="1:2">
-      <c r="A26" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B26" s="5" t="s">
+      <c r="D21" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" ht="30.75" spans="1:4">
+      <c r="A22" s="9" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="27" ht="32.25" spans="1:2">
-      <c r="A27" s="4" t="s">
+      <c r="B22" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="D22" s="13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="28" ht="32.25" spans="1:2">
-      <c r="A28" s="4" t="s">
+    <row r="23" spans="1:4">
+      <c r="A23" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B23" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="29" ht="32.25" spans="1:2">
-      <c r="A29" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="5" t="s">
+      <c r="D23" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="24" ht="30.75" spans="1:4">
+      <c r="A24" s="9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="30" ht="32.25" spans="1:2">
-      <c r="A30" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B30" s="5" t="s">
+      <c r="B24" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" s="10" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="31" ht="32.25" spans="1:2">
-      <c r="A31" s="4" t="s">
+      <c r="D24" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B25" s="12" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="32" ht="32.25" spans="1:2">
-      <c r="A32" s="4" t="s">
+      <c r="C25" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="D25" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="9" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="33" ht="32.25" spans="1:2">
-      <c r="A33" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B33" s="5" t="s">
+      <c r="B26" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="34" ht="32.25" spans="1:2">
-      <c r="A34" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B34" s="5" t="s">
+      <c r="D26" s="14"/>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="35" ht="32.25" spans="1:2">
-      <c r="A35" s="4" t="s">
+      <c r="B27" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="D27" s="14"/>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="9" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="36" ht="32.25" spans="1:2">
-      <c r="A36" s="4" t="s">
+      <c r="B28" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="D28" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="9" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="37" ht="32.25" spans="1:2">
-      <c r="A37" s="4" t="s">
+      <c r="B29" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="D29" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="9" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="38" ht="32.25" spans="1:2">
-      <c r="A38" s="4" t="s">
+      <c r="B30" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="D30" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="9" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="39" ht="32.25" spans="1:2">
-      <c r="A39" s="4" t="s">
+      <c r="B31" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="D31" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="32" ht="30.75" spans="1:4">
+      <c r="A32" s="9" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="40" ht="32.25" spans="1:2">
-      <c r="A40" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B40" s="5" t="s">
+      <c r="B32" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" s="10" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="41" ht="32.25" spans="1:2">
-      <c r="A41" s="4" t="s">
+      <c r="D32" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="B41" s="5" t="s">
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="9" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="42" ht="32.25" spans="1:2">
-      <c r="A42" s="4" t="s">
+      <c r="B33" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="D33" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="34" ht="30.75" spans="1:4">
+      <c r="A34" s="9" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="43" ht="32.25" spans="1:2">
-      <c r="A43" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B43" s="5" t="s">
+      <c r="B34" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="44" ht="32.25" spans="1:2">
-      <c r="A44" s="4" t="s">
+      <c r="D34" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B35" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="10" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="45" ht="32.25" spans="1:2">
-      <c r="A45" s="4" t="s">
+      <c r="D35" s="14"/>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B36" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="10" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="46" ht="32.25" spans="1:2">
-      <c r="A46" s="4" t="s">
+      <c r="D36" s="14"/>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B37" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" s="10" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="47" ht="32.25" spans="1:2">
-      <c r="A47" s="4" t="s">
+      <c r="D37" s="14"/>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B38" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" s="10" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="48" ht="32.25" spans="1:2">
-      <c r="A48" s="4" t="s">
+      <c r="D38" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B39" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="49" ht="32.25" spans="1:2">
-      <c r="A49" s="4" t="s">
+      <c r="D39" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B40" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C40" s="10" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="50" ht="32.25" spans="1:2">
-      <c r="A50" s="4" t="s">
+      <c r="D40" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B41" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C41" s="10" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="51" ht="32.25" spans="1:2">
-      <c r="A51" s="4" t="s">
+      <c r="D41" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B42" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" s="10" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="52" ht="32.25" spans="1:2">
-      <c r="A52" s="4" t="s">
+      <c r="D42" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B43" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" s="10" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="53" ht="32.25" spans="1:2">
-      <c r="A53" s="4" t="s">
+      <c r="D43" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B44" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44" s="10" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="54" ht="32.25" spans="1:2">
-      <c r="A54" s="4" t="s">
+      <c r="D44" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="45" ht="30.75" spans="1:4">
+      <c r="A45" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B45" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" s="10" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="55" ht="32.25" spans="1:2">
-      <c r="A55" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B55" s="5" t="s">
+      <c r="D45" s="13" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="56" ht="32.25" spans="1:2">
-      <c r="A56" s="4" t="s">
+    <row r="46" spans="1:4">
+      <c r="A46" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B46" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46" s="10" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="57" ht="32.25" spans="1:2">
-      <c r="A57" s="4" t="s">
+      <c r="D46" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="B47" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" s="10" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="58" ht="32.25" spans="1:2">
-      <c r="A58" s="6" t="s">
+      <c r="D47" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B48" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="10" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="59" ht="32.25" spans="1:2">
-      <c r="A59" s="4" t="s">
+      <c r="D48" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="B49" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C49" s="10" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="60" ht="32.25" spans="1:2">
-      <c r="A60" s="4" t="s">
+      <c r="D49" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B50" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50" s="10" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="61" ht="32.25" spans="1:2">
-      <c r="A61" s="4" t="s">
+      <c r="D50" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="B51" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C51" s="10" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="62" ht="32.25" spans="1:2">
-      <c r="A62" s="4" t="s">
+      <c r="D51" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="52" ht="30.75" spans="1:4">
+      <c r="A52" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="B52" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C52" s="10" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="63" ht="32.25" spans="1:2">
-      <c r="A63" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B63" s="5" t="s">
+      <c r="D52" s="13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="9" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="64" ht="32.25" spans="1:2">
-      <c r="A64" s="4" t="s">
+      <c r="B53" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C53" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="D53" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="9" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="65" ht="32.25" spans="1:2">
-      <c r="A65" s="4" t="s">
+      <c r="B54" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C54" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="D54" s="14"/>
+    </row>
+    <row r="55" ht="30.75" spans="1:4">
+      <c r="A55" s="9" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="66" ht="32.25" spans="1:2">
-      <c r="A66" s="4" t="s">
+      <c r="B55" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C55" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="D55" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="9" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="67" ht="32.25" spans="1:2">
-      <c r="A67" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B67" s="5" t="s">
+      <c r="B56" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="68" ht="32.25" spans="1:2">
-      <c r="A68" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B68" s="5" t="s">
+      <c r="D56" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="9" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="69" ht="32.25" spans="1:2">
-      <c r="A69" s="4" t="s">
+      <c r="B57" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C57" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="D57" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="9" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="70" ht="32.25" spans="1:2">
-      <c r="A70" s="4" t="s">
+      <c r="B58" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="D58" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="9" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="71" ht="32.25" spans="1:2">
-      <c r="A71" s="4" t="s">
+      <c r="B59" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C59" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="D59" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="9" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="72" ht="32.25" spans="1:2">
-      <c r="A72" s="4" t="s">
+      <c r="B60" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C60" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B72" s="5" t="s">
+      <c r="D60" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="9" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="73" ht="32.25" spans="1:2">
-      <c r="A73" s="4" t="s">
+      <c r="B61" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C61" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B73" s="5" t="s">
+      <c r="D61" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="9" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="74" ht="32.25" spans="1:2">
-      <c r="A74" s="4" t="s">
+      <c r="B62" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B74" s="5" t="s">
+      <c r="D62" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="9" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="75" ht="32.25" spans="1:2">
-      <c r="A75" s="4" t="s">
+      <c r="B63" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C63" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B75" s="5" t="s">
+      <c r="D63" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="9" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="76" ht="32.25" spans="1:2">
-      <c r="A76" s="4" t="s">
+      <c r="B64" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C64" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B76" s="5" t="s">
+      <c r="D64" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="9" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="77" ht="32.25" spans="1:2">
-      <c r="A77" s="4" t="s">
+      <c r="B65" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="D65" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="9" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="78" ht="32.25" spans="1:2">
-      <c r="A78" s="4" t="s">
+      <c r="B66" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C66" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="D66" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="9" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="79" ht="32.25" spans="1:2">
-      <c r="A79" s="4" t="s">
+      <c r="B67" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C67" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="D67" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="9" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="80" ht="32.25" spans="1:2">
-      <c r="A80" s="4" t="s">
+      <c r="B68" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C68" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="D68" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="9" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="81" ht="32.25" spans="1:2">
-      <c r="A81" s="4" t="s">
+      <c r="B69" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C69" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="D69" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="9" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="82" ht="32.25" spans="1:2">
-      <c r="A82" s="4" t="s">
+      <c r="B70" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C70" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="B82" s="5" t="s">
+      <c r="D70" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="9" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="83" ht="32.25" spans="1:2">
-      <c r="A83" s="4" t="s">
+      <c r="B71" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C71" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="D71" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="9" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="84" ht="32.25" spans="1:2">
-      <c r="A84" s="4" t="s">
+      <c r="B72" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C72" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="B84" s="5" t="s">
+      <c r="D72" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="9" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="85" ht="32.25" spans="1:2">
-      <c r="A85" s="4" t="s">
+      <c r="B73" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C73" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="B85" s="5" t="s">
+      <c r="D73" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" s="9" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="86" ht="32.25" spans="1:2">
-      <c r="A86" s="4" t="s">
+      <c r="B74" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C74" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="B86" s="5" t="s">
+      <c r="D74" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75" s="9" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="87" ht="32.25" spans="1:2">
-      <c r="A87" s="4" t="s">
+      <c r="B75" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C75" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="D75" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76" s="9" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="88" ht="32.25" spans="1:2">
-      <c r="A88" s="4" t="s">
+      <c r="B76" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C76" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="D76" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77" s="9" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="89" ht="32.25" spans="1:2">
-      <c r="A89" s="4" t="s">
+      <c r="B77" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C77" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B89" s="5" t="s">
+      <c r="D77" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" s="9" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="90" ht="32.25" spans="1:2">
-      <c r="A90" s="4" t="s">
+      <c r="B78" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C78" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="B90" s="5" t="s">
+      <c r="D78" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" s="9" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="91" ht="32.25" spans="1:2">
-      <c r="A91" s="4" t="s">
+      <c r="B79" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C79" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="B91" s="5" t="s">
+      <c r="D79" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" s="9" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="92" ht="32.25" spans="1:2">
-      <c r="A92" s="4" t="s">
+      <c r="B80" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C80" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="B92" s="5" t="s">
+      <c r="D80" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81" s="9" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="93" ht="32.25" spans="1:2">
-      <c r="A93" s="4" t="s">
+      <c r="B81" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C81" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="B93" s="5" t="s">
+      <c r="D81" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
+      <c r="A82" s="9" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="94" ht="32.25" spans="1:2">
-      <c r="A94" s="4" t="s">
+      <c r="B82" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C82" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="B94" s="5" t="s">
+      <c r="D82" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83" s="9" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="95" ht="32.25" spans="1:2">
-      <c r="A95" s="4" t="s">
+      <c r="B83" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C83" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="B95" s="5" t="s">
+      <c r="D83" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
+      <c r="A84" s="9" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="96" ht="32.25" spans="1:2">
-      <c r="A96" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B96" s="5" t="s">
+      <c r="B84" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C84" s="10" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="97" ht="48" spans="1:2">
-      <c r="A97" s="4" t="s">
+      <c r="D84" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="B97" s="5" t="s">
+      <c r="B85" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C85" s="10" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="98" ht="32.25" spans="1:2">
-      <c r="A98" s="4" t="s">
+      <c r="D85" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="B98" s="5" t="s">
+      <c r="B86" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C86" s="10" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="99" ht="32.25" spans="1:2">
-      <c r="A99" s="4" t="s">
+      <c r="D86" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
+      <c r="A87" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B99" s="5" t="s">
+      <c r="B87" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87" s="10" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="100" ht="32.25" spans="1:2">
-      <c r="A100" s="4" t="s">
+      <c r="D87" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="B100" s="5" t="s">
+      <c r="B88" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C88" s="10" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="101" ht="48" spans="1:2">
-      <c r="A101" s="4" t="s">
+      <c r="D88" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
+      <c r="A89" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B101" s="5" t="s">
+      <c r="B89" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C89" s="10" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="102" ht="32.25" spans="1:2">
-      <c r="A102" s="4" t="s">
+      <c r="D89" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="B102" s="5" t="s">
+      <c r="B90" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" s="10" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="103" ht="32.25" spans="1:2">
-      <c r="A103" s="4" t="s">
+      <c r="D90" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
+      <c r="A91" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="B103" s="5" t="s">
+      <c r="B91" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C91" s="10" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="104" ht="32.25" spans="1:2">
-      <c r="A104" s="4" t="s">
+      <c r="D91" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="B104" s="5" t="s">
+      <c r="B92" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C92" s="10" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="105" ht="32.25" spans="1:2">
-      <c r="A105" s="4" t="s">
+      <c r="D92" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="B105" s="5" t="s">
+      <c r="B93" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C93" s="10" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="106" ht="32.25" spans="1:2">
-      <c r="A106" s="4" t="s">
+      <c r="D93" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="B106" s="5" t="s">
+      <c r="B94" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C94" s="10" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="107" ht="32.25" spans="1:2">
-      <c r="A107" s="4" t="s">
+      <c r="D94" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B107" s="5" t="s">
+      <c r="B95" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C95" s="10" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="108" ht="32.25" spans="1:2">
-      <c r="A108" s="4" t="s">
+      <c r="D95" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="B108" s="5" t="s">
+      <c r="B96" s="10" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="109" ht="32.25" spans="1:2">
-      <c r="A109" s="4" t="s">
+      <c r="C96" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="B109" s="5" t="s">
+      <c r="D96" s="14"/>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" s="9" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="110" ht="32.25" spans="1:2">
-      <c r="A110" s="4" t="s">
+      <c r="B97" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C97" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="B110" s="5" t="s">
+      <c r="D97" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
+      <c r="A98" s="9" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="111" ht="32.25" spans="1:2">
-      <c r="A111" s="4" t="s">
+      <c r="B98" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C98" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="B111" s="5" t="s">
+      <c r="D98" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="99" ht="30.75" spans="1:4">
+      <c r="A99" s="9" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="112" ht="32.25" spans="1:2">
-      <c r="A112" s="4" t="s">
+      <c r="B99" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C99" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="B112" s="5" t="s">
+      <c r="D99" s="13" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="113" ht="32.25" spans="1:2">
-      <c r="A113" s="4" t="s">
+    <row r="100" ht="30.75" spans="1:4">
+      <c r="A100" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B113" s="5" t="s">
+      <c r="B100" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C100" s="10" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="114" ht="32.25" spans="1:2">
-      <c r="A114" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B114" s="5" t="s">
+      <c r="D100" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
+      <c r="A101" s="9" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="115" ht="32.25" spans="1:2">
-      <c r="A115" s="4" t="s">
+      <c r="B101" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C101" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="B115" s="5" t="s">
+      <c r="D101" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4">
+      <c r="A102" s="9" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="116" ht="32.25" spans="1:2">
-      <c r="A116" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="B116" s="5" t="s">
+      <c r="B102" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C102" s="10" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="117" ht="32.25" spans="1:2">
-      <c r="A117" s="4" t="s">
+      <c r="D102" s="14"/>
+    </row>
+    <row r="103" spans="1:4">
+      <c r="A103" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="B117" s="5" t="s">
+      <c r="B103" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C103" s="10" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="118" ht="32.25" spans="1:2">
-      <c r="A118" s="4" t="s">
+      <c r="D103" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
+      <c r="A104" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="B118" s="5" t="s">
+      <c r="B104" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C104" s="10" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="119" ht="32.25" spans="1:2">
-      <c r="A119" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B119" s="5" t="s">
+      <c r="D104" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="105" ht="30.75" spans="1:4">
+      <c r="A105" s="9" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="120" ht="32.25" spans="1:2">
-      <c r="A120" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B120" s="5" t="s">
+      <c r="B105" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C105" s="10" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="121" ht="32.25" spans="1:2">
-      <c r="A121" s="4" t="s">
+      <c r="D105" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="B121" s="5" t="s">
+    </row>
+    <row r="106" ht="30.75" spans="1:4">
+      <c r="A106" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="122" ht="48" spans="1:2">
-      <c r="A122" s="4" t="s">
+      <c r="B106" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C106" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="B122" s="5" t="s">
+      <c r="D106" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="107" ht="30.75" spans="1:4">
+      <c r="A107" s="9" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="123" ht="32.25" spans="1:2">
-      <c r="A123" s="4" t="s">
+      <c r="B107" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C107" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="B123" s="5" t="s">
+      <c r="D107" s="13" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="124" ht="48" spans="1:2">
-      <c r="A124" s="4" t="s">
+    <row r="108" spans="1:4">
+      <c r="A108" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="B124" s="5" t="s">
+      <c r="B108" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C108" s="10" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="125" ht="48" spans="1:2">
-      <c r="A125" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="B125" s="5" t="s">
+      <c r="D108" s="14"/>
+    </row>
+    <row r="109" spans="1:4">
+      <c r="A109" s="9" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="126" ht="32.25" spans="1:2">
-      <c r="A126" s="4" t="s">
+      <c r="B109" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C109" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="B126" s="5" t="s">
+      <c r="D109" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="110" ht="30.75" spans="1:4">
+      <c r="A110" s="9" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="127" ht="32.25" spans="1:2">
-      <c r="A127" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="B127" s="5" t="s">
+      <c r="B110" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C110" s="10" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="128" ht="32.25" spans="1:2">
-      <c r="A128" s="4" t="s">
+      <c r="D110" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
+      <c r="A111" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B128" s="5" t="s">
+      <c r="B111" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C111" s="10" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="129" ht="32.25" spans="1:2">
-      <c r="A129" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="B129" s="5" t="s">
+      <c r="D111" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
+      <c r="A112" s="9" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="130" ht="32.25" spans="1:2">
-      <c r="A130" s="4" t="s">
+      <c r="B112" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C112" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="B130" s="5" t="s">
+      <c r="D112" s="14"/>
+    </row>
+    <row r="113" spans="1:4">
+      <c r="A113" s="9" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="131" ht="32.25" spans="1:2">
-      <c r="A131" s="4" t="s">
+      <c r="B113" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C113" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="B131" s="5" t="s">
+      <c r="D113" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="114" ht="30.75" spans="1:4">
+      <c r="A114" s="9" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="132" ht="32.25" spans="1:2">
-      <c r="A132" s="4" t="s">
+      <c r="B114" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C114" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="B132" s="5" t="s">
+      <c r="D114" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
+      <c r="A115" s="9" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="133" ht="32.25" spans="1:2">
-      <c r="A133" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="B133" s="5" t="s">
+      <c r="B115" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C115" s="10" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="134" ht="32.25" spans="1:2">
-      <c r="A134" s="4" t="s">
+      <c r="D115" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
+      <c r="A116" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="B134" s="5" t="s">
+      <c r="B116" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C116" s="10" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="135" ht="32.25" spans="1:2">
-      <c r="A135" s="4" t="s">
+      <c r="D116" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
+      <c r="A117" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="B135" s="5" t="s">
+      <c r="B117" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C117" s="10" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="136" ht="32.25" spans="1:2">
-      <c r="A136" s="4" t="s">
+      <c r="D117" s="14"/>
+    </row>
+    <row r="118" ht="30.75" spans="1:4">
+      <c r="A118" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="B136" s="5" t="s">
+      <c r="B118" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C118" s="10" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="137" ht="32.25" spans="1:2">
-      <c r="A137" s="4" t="s">
+      <c r="D118" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
+      <c r="A119" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="B137" s="5" t="s">
+      <c r="B119" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C119" s="10" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="138" ht="32.25" spans="1:2">
-      <c r="A138" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="B138" s="5" t="s">
+      <c r="D119" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4">
+      <c r="A120" s="9" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="139" ht="32.25" spans="1:2">
-      <c r="A139" s="4" t="s">
+      <c r="B120" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C120" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="B139" s="5" t="s">
+      <c r="D120" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
+      <c r="A121" s="9" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="140" ht="32.25" spans="1:2">
-      <c r="A140" s="4" t="s">
+      <c r="B121" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C121" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="B140" s="5" t="s">
+      <c r="D121" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="122" ht="30.75" spans="1:4">
+      <c r="A122" s="9" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="141" ht="32.25" spans="1:2">
-      <c r="A141" s="4" t="s">
+      <c r="B122" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C122" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="B141" s="5" t="s">
+      <c r="D122" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
+      <c r="A123" s="9" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="142" ht="32.25" spans="1:2">
-      <c r="A142" s="4" t="s">
+      <c r="B123" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C123" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="B142" s="5" t="s">
+      <c r="D123" s="14"/>
+    </row>
+    <row r="124" spans="1:4">
+      <c r="A124" s="9" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="143" ht="32.25" spans="1:2">
-      <c r="A143" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="B143" s="5" t="s">
+      <c r="B124" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C124" s="10" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="144" ht="32.25" spans="1:2">
-      <c r="A144" s="4" t="s">
+      <c r="D124" s="14"/>
+    </row>
+    <row r="125" spans="1:4">
+      <c r="A125" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="B144" s="5" t="s">
+      <c r="B125" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C125" s="10" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="145" ht="32.25" spans="1:2">
-      <c r="A145" s="4" t="s">
+      <c r="D125" s="14"/>
+    </row>
+    <row r="126" spans="1:4">
+      <c r="A126" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="B145" s="5" t="s">
+      <c r="B126" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C126" s="10" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="146" ht="32.25" spans="1:2">
-      <c r="A146" s="4" t="s">
+      <c r="D126" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4">
+      <c r="A127" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="B146" s="5" t="s">
+      <c r="B127" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C127" s="10" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="147" ht="32.25" spans="1:2">
-      <c r="A147" s="4" t="s">
+      <c r="D127" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
+      <c r="A128" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="B147" s="5" t="s">
+      <c r="B128" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C128" s="10" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="148" ht="32.25" spans="1:2">
-      <c r="A148" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="B148" s="5" t="s">
+      <c r="D128" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4">
+      <c r="A129" s="9" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="149" ht="32.25" spans="1:2">
-      <c r="A149" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="B149" s="5" t="s">
+      <c r="B129" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C129" s="10" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="150" ht="32.25" spans="1:2">
-      <c r="A150" s="4" t="s">
+      <c r="D129" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4">
+      <c r="A130" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="B150" s="5" t="s">
+      <c r="B130" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C130" s="10" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="151" ht="32.25" spans="1:2">
-      <c r="A151" s="4" t="s">
+      <c r="D130" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
+      <c r="A131" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="B151" s="5" t="s">
+      <c r="B131" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C131" s="10" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="152" ht="32.25" spans="1:2">
-      <c r="A152" s="4" t="s">
+      <c r="D131" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
+      <c r="A132" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B152" s="5" t="s">
+      <c r="B132" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C132" s="10" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="153" ht="32.25" spans="1:2">
-      <c r="A153" s="4" t="s">
+      <c r="D132" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
+      <c r="A133" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="B153" s="5" t="s">
+      <c r="B133" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C133" s="10" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="154" ht="32.25" spans="1:2">
-      <c r="A154" s="4" t="s">
+      <c r="D133" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
+      <c r="A134" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="B154" s="5" t="s">
+      <c r="B134" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C134" s="10" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="155" ht="32.25" spans="1:2">
-      <c r="A155" s="4" t="s">
+      <c r="D134" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="B155" s="5" t="s">
+      <c r="B135" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C135" s="10" t="s">
         <v>282</v>
       </c>
+      <c r="D135" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="B136" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C136" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="D136" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="B137" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C137" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="D137" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4">
+      <c r="A138" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="B138" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C138" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="D138" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="B139" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C139" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="D139" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="B140" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C140" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="D140" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="B141" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C141" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="D141" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4">
+      <c r="A142" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="B142" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C142" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="D142" s="11">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4">
+      <c r="A143" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="B143" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C143" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="D143" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4">
+      <c r="A144" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="B144" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C144" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="D144" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5">
+      <c r="A145" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="B145" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C145" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="D145" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5">
+      <c r="A146" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="B146" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C146" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="D146" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5">
+      <c r="A147" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="B147" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C147" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="D147" s="14"/>
+    </row>
+    <row r="148" spans="1:5">
+      <c r="A148" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="B148" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C148" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="D148" s="11">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5">
+      <c r="A149" s="9" t="s">
+        <v>309</v>
+      </c>
+      <c r="B149" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C149" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="D149" s="14"/>
+    </row>
+    <row r="150" spans="1:5">
+      <c r="A150" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="B150" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C150" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="D150" s="14"/>
+    </row>
+    <row r="151" spans="1:5">
+      <c r="A151" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="B151" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C151" s="10" t="s">
+        <v>314</v>
+      </c>
+      <c r="D151" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="152" ht="16.5" spans="1:5">
+      <c r="A152" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="B152" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C152" s="10" t="s">
+        <v>316</v>
+      </c>
+      <c r="D152" s="14"/>
+      <c r="E152" s="16"/>
+    </row>
+    <row r="153" ht="16.5" spans="1:5">
+      <c r="A153" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="B153" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C153" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="D153" s="11">
+        <v>46177</v>
+      </c>
+      <c r="E153" s="16"/>
+    </row>
+    <row r="154" ht="16.5" spans="1:5">
+      <c r="A154" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="B154" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C154" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="D154" s="14"/>
+      <c r="E154" s="16"/>
+    </row>
+    <row r="155" ht="16.5" spans="1:5">
+      <c r="A155" s="9" t="s">
+        <v>321</v>
+      </c>
+      <c r="B155" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C155" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="D155" s="11">
+        <v>46177</v>
+      </c>
+      <c r="E155" s="16"/>
+    </row>
+    <row r="156" ht="16.5" spans="1:5">
+      <c r="A156" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="B156" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C156" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="D156" s="11">
+        <v>46238</v>
+      </c>
+      <c r="E156" s="16"/>
+    </row>
+    <row r="157" ht="16.5" spans="1:5">
+      <c r="A157" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="B157" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C157" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="D157" s="14"/>
+      <c r="E157" s="16"/>
+    </row>
+    <row r="158" ht="30.75" spans="1:5">
+      <c r="A158" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="B158" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C158" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="D158" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E158" s="16"/>
+    </row>
+    <row r="159" ht="30.75" spans="1:5">
+      <c r="A159" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="B159" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C159" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="D159" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E159" s="16"/>
+    </row>
+    <row r="160" ht="30.75" spans="1:5">
+      <c r="A160" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="B160" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C160" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="D160" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E160" s="16"/>
+    </row>
+    <row r="161" ht="16.5" spans="1:10">
+      <c r="A161" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="B161" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C161" s="10" t="s">
+        <v>336</v>
+      </c>
+      <c r="D161" s="11">
+        <v>46207</v>
+      </c>
+      <c r="E161" s="16"/>
+    </row>
+    <row r="162" ht="30.75" spans="1:10">
+      <c r="A162" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="B162" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C162" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="D162" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="E162" s="16"/>
+    </row>
+    <row r="163" ht="30.75" spans="1:10">
+      <c r="A163" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="B163" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C163" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="D163" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E163" s="16"/>
+    </row>
+    <row r="164" ht="30.75" spans="1:10">
+      <c r="A164" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="B164" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C164" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="D164" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E164" s="16"/>
+      <c r="J164" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="165" ht="16.5" spans="1:10">
+      <c r="A165" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="B165" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C165" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="D165" s="11">
+        <v>46146</v>
+      </c>
+      <c r="E165" s="16"/>
+    </row>
+    <row r="166" ht="16.5" spans="1:10">
+      <c r="A166" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="B166" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C166" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="D166" s="11">
+        <v>46146</v>
+      </c>
+      <c r="E166" s="16"/>
+    </row>
+    <row r="167" ht="30.75" spans="1:10">
+      <c r="A167" s="9" t="s">
+        <v>347</v>
+      </c>
+      <c r="B167" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C167" s="10" t="s">
+        <v>348</v>
+      </c>
+      <c r="D167" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E167" s="16"/>
+    </row>
+    <row r="168" ht="30.75" spans="1:10">
+      <c r="A168" s="9" t="s">
+        <v>349</v>
+      </c>
+      <c r="B168" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C168" s="10" t="s">
+        <v>350</v>
+      </c>
+      <c r="D168" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E168" s="16"/>
+    </row>
+    <row r="169" ht="30.75" spans="1:10">
+      <c r="A169" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="B169" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C169" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="D169" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E169" s="16"/>
+    </row>
+    <row r="170" ht="30.75" spans="1:10">
+      <c r="A170" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="B170" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C170" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="D170" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E170" s="16"/>
+    </row>
+    <row r="171" ht="30.75" spans="1:10">
+      <c r="A171" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="B171" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C171" s="10" t="s">
+        <v>356</v>
+      </c>
+      <c r="D171" s="13" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="172" ht="30.75" spans="1:10">
+      <c r="A172" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="B172" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C172" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="D172" s="13" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10">
+      <c r="A173" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="B173" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C173" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="D173" s="14"/>
+    </row>
+    <row r="174" spans="1:10">
+      <c r="A174" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="B174" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="C174" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D174" s="14"/>
+    </row>
+    <row r="175" spans="1:10">
+      <c r="A175" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="B175" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C175" s="10" t="s">
+        <v>364</v>
+      </c>
+      <c r="D175" s="14"/>
+    </row>
+    <row r="176" spans="1:10">
+      <c r="A176" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B176" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C176" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="D176" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4">
+      <c r="A177" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="B177" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C177" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="D177" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4">
+      <c r="A178" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="B178" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C178" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="D178" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4">
+      <c r="A179" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="B179" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C179" s="10" t="s">
+        <v>372</v>
+      </c>
+      <c r="D179" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4">
+      <c r="A180" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="B180" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C180" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="D180" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4">
+      <c r="A181" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="B181" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C181" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="D181" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4">
+      <c r="A182" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="B182" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C182" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="D182" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4">
+      <c r="A183" s="9" t="s">
+        <v>379</v>
+      </c>
+      <c r="B183" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C183" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="D183" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4">
+      <c r="A184" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="B184" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C184" s="10" t="s">
+        <v>382</v>
+      </c>
+      <c r="D184" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4">
+      <c r="A185" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="B185" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C185" s="10" t="s">
+        <v>384</v>
+      </c>
+      <c r="D185" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4">
+      <c r="A186" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="B186" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C186" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="D186" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4">
+      <c r="A187" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="B187" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C187" s="10" t="s">
+        <v>388</v>
+      </c>
+      <c r="D187" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4">
+      <c r="A188" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="B188" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C188" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="D188" s="11">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4">
+      <c r="A189" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="B189" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C189" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="D189" s="14"/>
+    </row>
+    <row r="190" ht="30.75" spans="1:4">
+      <c r="A190" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="B190" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C190" s="10" t="s">
+        <v>394</v>
+      </c>
+      <c r="D190" s="13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4">
+      <c r="A191" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="B191" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C191" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="D191" s="11">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="192" ht="30.75" spans="1:4">
+      <c r="A192" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="B192" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C192" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="D192" s="13" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4">
+      <c r="A193" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="B193" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C193" s="10" t="s">
+        <v>401</v>
+      </c>
+      <c r="D193" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4">
+      <c r="A194" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="B194" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C194" s="10" t="s">
+        <v>403</v>
+      </c>
+      <c r="D194" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4">
+      <c r="A195" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="B195" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C195" s="10" t="s">
+        <v>405</v>
+      </c>
+      <c r="D195" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4">
+      <c r="A196" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="B196" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C196" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="D196" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4">
+      <c r="A197" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="B197" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C197" s="10" t="s">
+        <v>409</v>
+      </c>
+      <c r="D197" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4">
+      <c r="A198" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="B198" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C198" s="10" t="s">
+        <v>411</v>
+      </c>
+      <c r="D198" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4">
+      <c r="A199" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="B199" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C199" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="D199" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4">
+      <c r="A200" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="B200" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C200" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="D200" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4">
+      <c r="A201" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="B201" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C201" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="D201" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="202" ht="30.75" spans="1:4">
+      <c r="A202" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="B202" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C202" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D202" s="13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4">
+      <c r="A203" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="B203" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C203" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="D203" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4">
+      <c r="A204" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="B204" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C204" s="10">
+        <v>329.227</v>
+      </c>
+      <c r="D204" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4">
+      <c r="A205" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="B205" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C205" s="10" t="s">
+        <v>424</v>
+      </c>
+      <c r="D205" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="206" ht="30.75" spans="1:4">
+      <c r="A206" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="B206" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C206" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="D206" s="13" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4">
+      <c r="A207" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="B207" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C207" s="10" t="s">
+        <v>428</v>
+      </c>
+      <c r="D207" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4">
+      <c r="A208" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="B208" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C208" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="D208" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4">
+      <c r="A209" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="B209" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C209" s="10" t="s">
+        <v>432</v>
+      </c>
+      <c r="D209" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4">
+      <c r="A210" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="B210" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C210" s="10" t="s">
+        <v>434</v>
+      </c>
+      <c r="D210" s="11">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4">
+      <c r="A211" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="B211" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C211" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="D211" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4">
+      <c r="A212" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="B212" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C212" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="D212" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4">
+      <c r="A213" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="B213" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C213" s="10" t="s">
+        <v>440</v>
+      </c>
+      <c r="D213" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4">
+      <c r="A214" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="B214" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C214" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="D214" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4">
+      <c r="A215" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="B215" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C215" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="D215" s="11">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4">
+      <c r="A216" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="B216" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C216" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D216" s="11">
+        <v>46146</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:E151" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>